<commit_message>
beta v0.10.44: tsunami boss-style aim preview, shockwave 22, slower scissors, dodge i-frames
- Tsunami aim preview: red front line across the wave width plus a red band
  fading forward over the sweep length
- Shockwave base damage 15 -> 22
- Scissors rest between attacks 0.6-1.1s -> 0.8-1.35s (def.gap)
- Perfect dodge grants 0.5s invulnerability

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -3261,7 +3261,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">15
+      <t xml:space="preserve">22
 </t>
     </r>
     <r>
@@ -3378,7 +3378,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">15 </t>
+      <t xml:space="preserve">22 </t>
     </r>
     <r>
       <rPr>
@@ -11406,6 +11406,24 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1.5
+gap</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[0.8, 1.35]
 evolve</t>
     </r>
     <r>
@@ -32878,7 +32896,7 @@
       </c>
       <c r="P13" s="10"/>
     </row>
-    <row r="14" customFormat="false" ht="161.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="174.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
         <v>346</v>
       </c>

</xml_diff>

<commit_message>
beta v0.10.47: red-ink execute targets bosses first, then elites, within range
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -7427,7 +7427,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">對目標附近最近的敵人造成 </t>
+      <t xml:space="preserve">對目標範圍內的敵人造成 </t>
     </r>
     <r>
       <rPr>
@@ -7444,7 +7444,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">點毀滅性傷害。</t>
+      <t xml:space="preserve">點毀滅性傷害：優先頭目，其次菁英怪，再來才是最近的敵人。</t>
     </r>
   </si>
   <si>

</xml_diff>

<commit_message>
v0.11.07: chalk trajectory, grid meters, per-page whiteout, NPC colliders, ult FX
- Chalk throws show a trajectory telegraph and fly along it
- Distances in card and relic text use floor grid meters
- Whiteout relic rearms on every page
- Restore NPC colliders lost in v0.11.04
- Ult cut-ins gain an ink iris, rotating rays, a marquee band, impact
  shockwaves with cracks, screen quake and a card shine

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -1502,7 +1502,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內造成最多 </t>
+      <t xml:space="preserve">公尺內造成最多 </t>
     </r>
     <r>
       <rPr>
@@ -1546,7 +1546,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內造成最多 </t>
+      <t xml:space="preserve">公尺內造成最多 </t>
     </r>
     <r>
       <rPr>
@@ -2042,7 +2042,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">的路徑，長出一道擋住敵彈的牆，持續 </t>
+      <t xml:space="preserve">公尺的路徑，長出一道擋住敵彈的牆，持續 </t>
     </r>
     <r>
       <rPr>
@@ -2086,7 +2086,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">的路徑，長出一道擋住敵彈的牆，持續 </t>
+      <t xml:space="preserve">公尺的路徑，長出一道擋住敵彈的牆，持續 </t>
     </r>
     <r>
       <rPr>
@@ -3507,7 +3507,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內的敵人並造成 </t>
+      <t xml:space="preserve">公尺內的敵人並造成 </t>
     </r>
     <r>
       <rPr>
@@ -3551,7 +3551,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內的敵人並造成 </t>
+      <t xml:space="preserve">公尺內的敵人並造成 </t>
     </r>
     <r>
       <rPr>
@@ -4671,7 +4671,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內的敵人都受到 </t>
+      <t xml:space="preserve">公尺內的敵人都受到 </t>
     </r>
     <r>
       <rPr>
@@ -4715,7 +4715,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內的敵人都受到 </t>
+      <t xml:space="preserve">公尺內的敵人都受到 </t>
     </r>
     <r>
       <rPr>
@@ -4864,7 +4864,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內造成 </t>
+      <t xml:space="preserve">公尺內造成 </t>
     </r>
     <r>
       <rPr>
@@ -4908,7 +4908,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內造成 </t>
+      <t xml:space="preserve">公尺內造成 </t>
     </r>
     <r>
       <rPr>
@@ -5083,7 +5083,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內的所有敵彈，每吸 </t>
+      <t xml:space="preserve">公尺內的所有敵彈，每吸 </t>
     </r>
     <r>
       <rPr>
@@ -5161,7 +5161,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內的所有敵彈，每吸 </t>
+      <t xml:space="preserve">公尺內的所有敵彈，每吸 </t>
     </r>
     <r>
       <rPr>
@@ -5584,7 +5584,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內的敵人釘在原地 </t>
+      <t xml:space="preserve">公尺內的敵人釘在原地 </t>
     </r>
     <r>
       <rPr>
@@ -5645,7 +5645,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內的敵人釘在原地 </t>
+      <t xml:space="preserve">公尺內的敵人釘在原地 </t>
     </r>
     <r>
       <rPr>
@@ -5970,7 +5970,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">後折返；去程與回程各對路徑上的敵人造成 </t>
+      <t xml:space="preserve">公尺後折返；去程與回程各對路徑上的敵人造成 </t>
     </r>
     <r>
       <rPr>
@@ -6014,7 +6014,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">後折返；去程與回程各對路徑上的敵人造成 </t>
+      <t xml:space="preserve">公尺後折返；去程與回程各對路徑上的敵人造成 </t>
     </r>
     <r>
       <rPr>
@@ -6989,7 +6989,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">的墨刺地，</t>
+      <t xml:space="preserve">公尺的墨刺地，</t>
     </r>
     <r>
       <rPr>
@@ -7050,7 +7050,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">的墨刺地，</t>
+      <t xml:space="preserve">公尺的墨刺地，</t>
     </r>
     <r>
       <rPr>
@@ -8156,7 +8156,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">內的敵人吸過來，</t>
+      <t xml:space="preserve">公尺內的敵人吸過來，</t>
     </r>
     <r>
       <rPr>
@@ -27056,7 +27056,7 @@
     <t xml:space="preserve">立可白</t>
   </si>
   <si>
-    <t xml:space="preserve">每局第一次受到傷害時，完全抵銷這次傷害。</t>
+    <t xml:space="preserve">每一頁（每個房間）第一次受到傷害時，完全抵銷這次傷害。</t>
   </si>
   <si>
     <r>
@@ -27466,7 +27466,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3 </t>
+      <t xml:space="preserve">1.5 </t>
     </r>
     <r>
       <rPr>
@@ -29351,7 +29351,47 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">0.7
+      <t xml:space="preserve">0.85
+teleLen</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">16
+teleW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.22
 dashCd</t>
     </r>
     <r>
@@ -36110,7 +36150,7 @@
       </c>
       <c r="G4" s="10"/>
     </row>
-    <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
         <v>786</v>
       </c>

</xml_diff>

<commit_message>
beta v0.11.08: richer ult cut-in FX, clear low-HP vignette on menu, dodge goal 3, weapon page without dice
- Ult cut-in: drop the red marquee band; add brush slashes, card afterimages, motif zoom punch, halftone ring, ink droplets and paper scraps at impact
- Leaving a run at low HP no longer carries the red edge vignette into the main menu
- Discipline course goal is now 3 chalk dodges; course text describes the trajectory telegraph
- Weapon screen drops the outfit randomizer button, leaving equip and back only

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -29106,7 +29106,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">秒老師從附近丟一支粉筆過來（出手前地上先出現紅圈）
+      <t xml:space="preserve">秒老師從附近丟一支粉筆過來（出手前先畫出粉筆的飛行軌跡）
 • 衝刺冷卻 −</t>
     </r>
     <r>
@@ -29431,7 +29431,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">4</t>
+      <t xml:space="preserve">3</t>
     </r>
   </si>
   <si>

</xml_diff>

<commit_message>
beta v0.12.03: slingshot weapon and weapon unlock sync
Add the 橡皮筋彈弓 charge weapon (hold to charge, release to fire, piercing, charge bar HUD, move slow while charging) with codex anim, sound and model. Rebalance weapon unlock levels (stapler 7, highlighter 9, compass 12, crayon 15, slingshot 18), gate all weapon pickers by level, auto-swap a locked last weapon with a one-time toast, and list weapons in the level view.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1323" uniqueCount="909">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1326" uniqueCount="912">
   <si>
     <r>
       <rPr>
@@ -12799,7 +12799,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">。使用圓規時不會出現（抽到直接棄掉）。</t>
+      <t xml:space="preserve">。使用圓規或橡皮筋彈弓時不會出現（抽到直接棄掉）。</t>
     </r>
   </si>
   <si>
@@ -18263,6 +18263,15 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">slingshot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">橡皮筋彈弓</t>
+  </si>
+  <si>
+    <t xml:space="preserve">蓄力穿透・無彈匣</t>
+  </si>
+  <si>
     <t xml:space="preserve">id</t>
   </si>
   <si>
@@ -31203,6 +31212,24 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">reload</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.9
+charge</t>
     </r>
     <r>
       <rPr>
@@ -38621,7 +38648,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O8"/>
+  <dimension ref="A1:O9"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -38828,7 +38855,7 @@
         <v>499</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>500</v>
@@ -38874,7 +38901,7 @@
         <v>503</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>504</v>
@@ -38920,7 +38947,7 @@
         <v>506</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>507</v>
@@ -38966,7 +38993,7 @@
         <v>510</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>511</v>
@@ -39003,6 +39030,50 @@
         <v>512</v>
       </c>
       <c r="O8" s="10"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>513</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>514</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>515</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J9" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="L9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="7" t="n">
+        <f aca="false">ROUND(E9*F9/G9,1)</f>
+        <v>150</v>
+      </c>
+      <c r="N9" s="7"/>
+      <c r="O9" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -39032,19 +39103,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -39052,325 +39123,325 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>82</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="377.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="F19" s="10"/>
     </row>
@@ -39405,13 +39476,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -39419,13 +39490,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="D2" s="16" t="n">
         <f aca="false">ROUND(B2/SUM(B$2:B$13),3)</f>
@@ -39435,13 +39506,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">ROUND(B3/SUM(B$2:B$13),3)</f>
@@ -39451,13 +39522,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="D4" s="16" t="n">
         <f aca="false">ROUND(B4/SUM(B$2:B$13),3)</f>
@@ -39467,13 +39538,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">ROUND(B5/SUM(B$2:B$13),3)</f>
@@ -39483,13 +39554,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="D6" s="16" t="n">
         <f aca="false">ROUND(B6/SUM(B$2:B$13),3)</f>
@@ -39499,13 +39570,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="D7" s="16" t="n">
         <f aca="false">ROUND(B7/SUM(B$2:B$13),3)</f>
@@ -39515,13 +39586,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">ROUND(B8/SUM(B$2:B$13),3)</f>
@@ -39531,13 +39602,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">ROUND(B9/SUM(B$2:B$13),3)</f>
@@ -39547,13 +39618,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">ROUND(B10/SUM(B$2:B$13),3)</f>
@@ -39563,13 +39634,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">ROUND(B11/SUM(B$2:B$13),3)</f>
@@ -39579,13 +39650,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">ROUND(B12/SUM(B$2:B$13),3)</f>
@@ -39595,13 +39666,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">ROUND(B13/SUM(B$2:B$13),3)</f>
@@ -39611,13 +39682,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">ROUND(B14/SUM(B$14:B$22),3)</f>
@@ -39627,13 +39698,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">ROUND(B15/SUM(B$14:B$22),3)</f>
@@ -39643,13 +39714,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="D16" s="16" t="n">
         <f aca="false">ROUND(B16/SUM(B$14:B$22),3)</f>
@@ -39659,13 +39730,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">ROUND(B17/SUM(B$14:B$22),3)</f>
@@ -39675,13 +39746,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">ROUND(B18/SUM(B$14:B$22),3)</f>
@@ -39691,13 +39762,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">ROUND(B19/SUM(B$14:B$22),3)</f>
@@ -39707,13 +39778,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">ROUND(B20/SUM(B$14:B$22),3)</f>
@@ -39723,13 +39794,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="B21" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="D21" s="16" t="n">
         <f aca="false">ROUND(B21/SUM(B$14:B$22),3)</f>
@@ -39739,13 +39810,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="B22" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="D22" s="16" t="n">
         <f aca="false">ROUND(B22/SUM(B$14:B$22),3)</f>
@@ -39781,16 +39852,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -39798,13 +39869,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>2</v>
@@ -39813,13 +39884,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>5</v>
@@ -39828,13 +39899,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>25</v>
@@ -39843,13 +39914,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>1</v>
@@ -39858,13 +39929,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>10</v>
@@ -39873,13 +39944,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2.5</v>
@@ -39888,13 +39959,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>5</v>
@@ -39903,13 +39974,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>2</v>
@@ -39918,13 +39989,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>0.35</v>
@@ -39933,13 +40004,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>5</v>
@@ -39948,13 +40019,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>1</v>
@@ -39963,28 +40034,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="E13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>0.2</v>
@@ -39993,28 +40064,28 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
       <c r="E15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>1</v>
@@ -40023,10 +40094,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
@@ -40036,13 +40107,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>5</v>
@@ -40051,10 +40122,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
@@ -40064,10 +40135,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
@@ -40077,10 +40148,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
@@ -40090,13 +40161,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>60000</v>
@@ -40105,13 +40176,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="D23" s="8" t="n">
         <v>45000</v>
@@ -40120,13 +40191,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>35000</v>
@@ -40135,13 +40206,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="D25" s="8" t="n">
         <v>20000</v>
@@ -40150,13 +40221,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>10000</v>
@@ -40165,13 +40236,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="D27" s="8" t="n">
         <v>5000</v>
@@ -40180,13 +40251,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>60000</v>
@@ -40195,13 +40266,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="D29" s="8" t="n">
         <v>45000</v>
@@ -40210,13 +40281,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>35000</v>
@@ -40225,13 +40296,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="D31" s="8" t="n">
         <v>20000</v>
@@ -40240,13 +40311,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>10000</v>
@@ -40255,13 +40326,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="D33" s="8" t="n">
         <v>5000</v>
@@ -40270,616 +40341,616 @@
     </row>
     <row r="34" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="E34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="E35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="E36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
       <c r="E37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="E38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="E39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="E40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B41" s="7" t="s">
+        <v>719</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>720</v>
+      </c>
+      <c r="D41" s="8" t="s">
         <v>716</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>717</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>713</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="D43" s="8" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="E43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="E44" s="10"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="E45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="E46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="E47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>731</v>
+        <v>734</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="E48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="E49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="E50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="E51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="E52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="E53" s="10"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="E54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>749</v>
+        <v>752</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="E55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>753</v>
+        <v>756</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="E56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="E57" s="10"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="E58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="E59" s="10"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="E60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>766</v>
+        <v>769</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="E61" s="10"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>768</v>
+        <v>771</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>769</v>
+        <v>772</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="E62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>772</v>
+        <v>775</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>773</v>
+        <v>776</v>
       </c>
       <c r="E63" s="10"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>774</v>
+        <v>777</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>775</v>
+        <v>778</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="E64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>777</v>
+        <v>780</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>778</v>
+        <v>781</v>
       </c>
       <c r="E65" s="10"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>779</v>
+        <v>782</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>780</v>
+        <v>783</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="E66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>781</v>
+        <v>784</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="E67" s="10"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>783</v>
+        <v>786</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>784</v>
+        <v>787</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>785</v>
+        <v>788</v>
       </c>
       <c r="E68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>786</v>
+        <v>789</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>787</v>
+        <v>790</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="E69" s="10"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>790</v>
+        <v>793</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>791</v>
+        <v>794</v>
       </c>
       <c r="E70" s="10"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>792</v>
+        <v>795</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>793</v>
+        <v>796</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>794</v>
+        <v>797</v>
       </c>
       <c r="E71" s="10"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>795</v>
+        <v>798</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="E72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>798</v>
+        <v>801</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>799</v>
+        <v>802</v>
       </c>
       <c r="E73" s="10"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>800</v>
+        <v>803</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>801</v>
+        <v>804</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>802</v>
+        <v>805</v>
       </c>
       <c r="E74" s="10"/>
     </row>
@@ -40911,19 +40982,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>803</v>
+        <v>806</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>804</v>
+        <v>807</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>805</v>
+        <v>808</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>806</v>
+        <v>809</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -40931,370 +41002,370 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>808</v>
+        <v>811</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>810</v>
+        <v>813</v>
       </c>
       <c r="F2" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>811</v>
+        <v>814</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>812</v>
+        <v>815</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>813</v>
+        <v>816</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>814</v>
+        <v>817</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>815</v>
+        <v>818</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>816</v>
+        <v>819</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>817</v>
+        <v>820</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>818</v>
+        <v>821</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>820</v>
+        <v>823</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>821</v>
+        <v>824</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>822</v>
+        <v>825</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>823</v>
+        <v>826</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>824</v>
+        <v>827</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>825</v>
+        <v>828</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>826</v>
+        <v>829</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>827</v>
+        <v>830</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>828</v>
+        <v>831</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>829</v>
+        <v>832</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>830</v>
+        <v>833</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>832</v>
+        <v>835</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>833</v>
+        <v>836</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>834</v>
+        <v>837</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>835</v>
+        <v>838</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>836</v>
+        <v>839</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>837</v>
+        <v>840</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>838</v>
+        <v>841</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>839</v>
+        <v>842</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>840</v>
+        <v>843</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>841</v>
+        <v>844</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>842</v>
+        <v>845</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>843</v>
+        <v>846</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>844</v>
+        <v>847</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>845</v>
+        <v>848</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>846</v>
+        <v>849</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>847</v>
+        <v>850</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>848</v>
+        <v>851</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>849</v>
+        <v>852</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>850</v>
+        <v>853</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>851</v>
+        <v>854</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>852</v>
+        <v>855</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>853</v>
+        <v>856</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>854</v>
+        <v>857</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>855</v>
+        <v>858</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>856</v>
+        <v>859</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>857</v>
+        <v>860</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>858</v>
+        <v>861</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>859</v>
+        <v>862</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>833</v>
+        <v>836</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>860</v>
+        <v>863</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>861</v>
+        <v>864</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>862</v>
+        <v>865</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>863</v>
+        <v>866</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>864</v>
+        <v>867</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>865</v>
+        <v>868</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>866</v>
+        <v>869</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>867</v>
+        <v>870</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>868</v>
+        <v>871</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>869</v>
+        <v>872</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>870</v>
+        <v>873</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>871</v>
+        <v>874</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>872</v>
+        <v>875</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="7" t="n">
@@ -41333,22 +41404,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>874</v>
+        <v>877</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>487</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>875</v>
+        <v>878</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>876</v>
+        <v>879</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>806</v>
+        <v>809</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -41356,115 +41427,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>877</v>
+        <v>880</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>878</v>
+        <v>881</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>879</v>
+        <v>882</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>880</v>
+        <v>883</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>881</v>
+        <v>884</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>883</v>
+        <v>886</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>884</v>
+        <v>887</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>885</v>
+        <v>888</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>886</v>
+        <v>889</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>887</v>
+        <v>890</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>888</v>
+        <v>891</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>889</v>
+        <v>892</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>890</v>
+        <v>893</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>891</v>
+        <v>894</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>892</v>
+        <v>895</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>893</v>
+        <v>896</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>894</v>
+        <v>897</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>895</v>
+        <v>898</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>896</v>
+        <v>899</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>897</v>
+        <v>900</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>898</v>
+        <v>901</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>899</v>
+        <v>902</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>900</v>
+        <v>903</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>901</v>
+        <v>904</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>902</v>
+        <v>905</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>903</v>
+        <v>906</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>904</v>
+        <v>907</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>905</v>
+        <v>908</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>906</v>
+        <v>909</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>907</v>
+        <v>910</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>908</v>
+        <v>911</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
beta v0.12.05: slingshot pull, active effects bar, ult cut-in rework, trap model
Slingshot gets a band pull-back animation and doubled timings (2s full charge), cast cards with lasting effects show in a new active-effects bar, training info shrinks to three text lines, four-way shot aims with four lines, ult cut-ins drop the shared generic effects and hand the skill icon off to where it lands, bear trap is rebuilt with a snap animation, redraw slides cards away and refills faster, box fort boxes break in one hit from any weapon, and the weapon page jumps to the equipped weapon.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -6310,18 +6310,18 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">抵擋次數：</t>
+      <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">數量：</t>
     </r>
     <r>
       <rPr>
@@ -6358,24 +6358,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">個紙箱，每個 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">點耐久，可以擋下敵彈；打破時 </t>
+      <t xml:space="preserve">個紙箱，可以擋下敵彈；任何武器或敵彈打一下就會破。打破時 </t>
     </r>
     <r>
       <rPr>
@@ -6479,23 +6462,6 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個紙箱，每個 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
       <t xml:space="preserve">4 </t>
     </r>
     <r>
@@ -6504,7 +6470,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">點耐久，可以擋下敵彈；打破時 </t>
+      <t xml:space="preserve">個紙箱，可以擋下敵彈；任何武器或敵彈打一下就會破。打破時 </t>
     </r>
     <r>
       <rPr>
@@ -36035,12 +36001,14 @@
         <v>36</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>117</v>
+        <v>37</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G33" s="8"/>
+        <v>38</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>12</v>
+      </c>
       <c r="H33" s="8" t="n">
         <v>12</v>
       </c>

</xml_diff>

<commit_message>
beta v0.12.07: 1.7s slingshot, stronger ult impact, 3 cards per early level
Slingshot full charge is now 1.7s. Ult cut-ins regain screen impact: tinted rays, speed lines, shockwaves, cracks, halftone, ink drops and paper scraps return, plus a burst of the skill's own icon at impact and again where it lands, and an in-world flash, double ring and splash at the cast point. Levels 2-5 now each unlock three cards (mini shield moves to 3, spare magazine to 4).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -3748,6 +3748,238 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">miniShield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">小紙盾</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">抵擋次數：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">持續</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">獲得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">片紙盾，持續 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒（可以和其他紙盾疊加）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">獲得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">片紙盾，持續 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒（可以和其他紙盾疊加）。</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">mark</t>
   </si>
   <si>
@@ -4282,6 +4514,73 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">spareMag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">備用彈匣</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">redraw</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">立刻補滿彈匣（螢光筆熱度歸零，圓規重置投擲冷卻），並增加 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次重抽次數。</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">（同基本）</t>
+  </si>
+  <si>
     <t xml:space="preserve">clone</t>
   </si>
   <si>
@@ -5859,238 +6158,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">miniShield</t>
-  </si>
-  <si>
-    <t xml:space="preserve">小紙盾</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">抵擋次數：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">持續</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">獲得 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">片紙盾，持續 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒（可以和其他紙盾疊加）。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">獲得 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">片紙盾，持續 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒（可以和其他紙盾疊加）。</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">paperBlade</t>
   </si>
   <si>
@@ -7610,73 +7677,6 @@
       </rPr>
       <t xml:space="preserve">傷害。</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">spareMag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">備用彈匣</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">redraw</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">立刻補滿彈匣（螢光筆熱度歸零，圓規重置投擲冷卻），並增加 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次重抽次數。</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">（同基本）</t>
   </si>
   <si>
     <t xml:space="preserve">reflect</t>
@@ -35139,7 +35139,7 @@
       </c>
       <c r="P14" s="10"/>
     </row>
-    <row r="15" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
         <v>128</v>
       </c>
@@ -35150,19 +35150,17 @@
         <v>35</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>130</v>
+        <v>97</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>131</v>
+        <v>67</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G15" s="8" t="n">
-        <v>14</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G15" s="8"/>
       <c r="H15" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I15" s="8" t="n">
         <v>0</v>
@@ -35174,39 +35172,41 @@
         <v>1</v>
       </c>
       <c r="L15" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="M15" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="N15" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="M15" s="9" t="s">
+      <c r="O15" s="7" t="s">
         <v>133</v>
-      </c>
-      <c r="N15" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="O15" s="7" t="s">
-        <v>135</v>
       </c>
       <c r="P15" s="10"/>
     </row>
-    <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>67</v>
+        <v>137</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G16" s="8"/>
+        <v>60</v>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>14</v>
+      </c>
       <c r="H16" s="8" t="n">
         <v>4</v>
       </c>
@@ -35225,10 +35225,10 @@
       <c r="M16" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="N16" s="6" t="s">
+      <c r="N16" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="O16" s="6" t="s">
+      <c r="O16" s="7" t="s">
         <v>141</v>
       </c>
       <c r="P16" s="10"/>
@@ -35244,303 +35244,297 @@
         <v>35</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>144</v>
+        <v>67</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G17" s="8" t="n">
-        <v>8</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G17" s="8"/>
       <c r="H17" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I17" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J17" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L17" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="M17" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="M17" s="9" t="s">
+      <c r="N17" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="N17" s="7" t="s">
+      <c r="O17" s="6" t="s">
         <v>147</v>
-      </c>
-      <c r="O17" s="7" t="s">
-        <v>148</v>
       </c>
       <c r="P17" s="10"/>
     </row>
-    <row r="18" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>149</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>150</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>36</v>
+        <v>136</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>151</v>
+        <v>67</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G18" s="8" t="n">
-        <v>11</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G18" s="8"/>
       <c r="H18" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I18" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="L18" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="L18" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="M18" s="8"/>
+      <c r="N18" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="O18" s="7" t="s">
         <v>152</v>
-      </c>
-      <c r="M18" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="N18" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="O18" s="7" t="s">
-        <v>155</v>
       </c>
       <c r="P18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>74</v>
+        <v>136</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>90</v>
+        <v>155</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>60</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I19" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K19" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L19" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="M19" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="N19" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="M19" s="9" t="s">
+      <c r="O19" s="7" t="s">
         <v>159</v>
-      </c>
-      <c r="N19" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="O19" s="7" t="s">
-        <v>161</v>
       </c>
       <c r="P19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>97</v>
+        <v>36</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>117</v>
+        <v>162</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>164</v>
-      </c>
-      <c r="G20" s="8"/>
+        <v>60</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>11</v>
+      </c>
       <c r="H20" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I20" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L20" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="M20" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="N20" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="M20" s="9" t="s">
+      <c r="O20" s="7" t="s">
         <v>166</v>
-      </c>
-      <c r="N20" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="O20" s="7" t="s">
-        <v>168</v>
       </c>
       <c r="P20" s="10"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>130</v>
+        <v>74</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>171</v>
+        <v>90</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G21" s="8"/>
+        <v>60</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>10</v>
+      </c>
       <c r="H21" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I21" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K21" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L21" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="M21" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="N21" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="O21" s="7" t="s">
         <v>172</v>
-      </c>
-      <c r="M21" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="N21" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="O21" s="7" t="s">
-        <v>175</v>
       </c>
       <c r="P21" s="10"/>
     </row>
-    <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>130</v>
+        <v>97</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G22" s="8" t="n">
-        <v>12</v>
-      </c>
+        <v>175</v>
+      </c>
+      <c r="G22" s="8"/>
       <c r="H22" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I22" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="M22" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="N22" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="M22" s="9" t="s">
+      <c r="O22" s="7" t="s">
         <v>179</v>
-      </c>
-      <c r="N22" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="O22" s="7" t="s">
-        <v>181</v>
       </c>
       <c r="P22" s="10"/>
     </row>
-    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C23" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>97</v>
+        <v>136</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>59</v>
+        <v>182</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G23" s="8" t="n">
-        <v>8</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G23" s="8"/>
       <c r="H23" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I23" s="8" t="n">
         <v>0</v>
@@ -35552,131 +35546,133 @@
         <v>3</v>
       </c>
       <c r="L23" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="M23" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="M23" s="9" t="s">
+      <c r="N23" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="N23" s="7" t="s">
+      <c r="O23" s="7" t="s">
         <v>186</v>
-      </c>
-      <c r="O23" s="7" t="s">
-        <v>187</v>
       </c>
       <c r="P23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>188</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>189</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>97</v>
+        <v>136</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>67</v>
+        <v>137</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G24" s="8"/>
+        <v>60</v>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>12</v>
+      </c>
       <c r="H24" s="8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I24" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L24" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="M24" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="M24" s="9" t="s">
+      <c r="N24" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="N24" s="7" t="s">
+      <c r="O24" s="7" t="s">
         <v>192</v>
-      </c>
-      <c r="O24" s="7" t="s">
-        <v>193</v>
       </c>
       <c r="P24" s="10"/>
     </row>
     <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>194</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>195</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>36</v>
+        <v>97</v>
       </c>
       <c r="E25" s="7" t="s">
         <v>59</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I25" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J25" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K25" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L25" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="M25" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="M25" s="9" t="s">
+      <c r="N25" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="N25" s="7" t="s">
+      <c r="O25" s="7" t="s">
         <v>198</v>
-      </c>
-      <c r="O25" s="7" t="s">
-        <v>199</v>
       </c>
       <c r="P25" s="10"/>
     </row>
-    <row r="26" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>200</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>201</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>9</v>
@@ -35688,93 +35684,93 @@
         <v>0</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L26" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="M26" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="M26" s="9" t="s">
+      <c r="N26" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="N26" s="7" t="s">
+      <c r="O26" s="7" t="s">
         <v>204</v>
-      </c>
-      <c r="O26" s="7" t="s">
-        <v>205</v>
       </c>
       <c r="P26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="B27" s="7" t="s">
         <v>206</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>207</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>208</v>
+        <v>90</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G27" s="8"/>
+        <v>60</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>9</v>
+      </c>
       <c r="H27" s="8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I27" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L27" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="M27" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="N27" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="M27" s="9" t="s">
+      <c r="O27" s="7" t="s">
         <v>210</v>
-      </c>
-      <c r="N27" s="7" t="s">
-        <v>211</v>
-      </c>
-      <c r="O27" s="7" t="s">
-        <v>212</v>
       </c>
       <c r="P27" s="10"/>
     </row>
     <row r="28" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>90</v>
+        <v>213</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="G28" s="8" t="n">
-        <v>9</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G28" s="8"/>
       <c r="H28" s="8" t="n">
         <v>10</v>
       </c>
@@ -35788,88 +35784,88 @@
         <v>2</v>
       </c>
       <c r="L28" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="M28" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="M28" s="9" t="s">
+      <c r="N28" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="N28" s="7" t="s">
+      <c r="O28" s="7" t="s">
         <v>217</v>
-      </c>
-      <c r="O28" s="7" t="s">
-        <v>218</v>
       </c>
       <c r="P28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="B29" s="7" t="s">
         <v>219</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>220</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>151</v>
+        <v>90</v>
       </c>
       <c r="F29" s="7" t="s">
         <v>60</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I29" s="8" t="n">
         <v>0</v>
       </c>
       <c r="J29" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L29" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="M29" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="M29" s="9" t="s">
+      <c r="N29" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="N29" s="7" t="s">
+      <c r="O29" s="7" t="s">
         <v>223</v>
-      </c>
-      <c r="O29" s="7" t="s">
-        <v>224</v>
       </c>
       <c r="P29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="B30" s="7" t="s">
         <v>225</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>226</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>90</v>
+        <v>162</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>60</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="H30" s="8" t="n">
         <v>11</v>
@@ -35878,45 +35874,47 @@
         <v>0</v>
       </c>
       <c r="J30" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K30" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L30" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="M30" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="M30" s="9" t="s">
+      <c r="N30" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="N30" s="7" t="s">
+      <c r="O30" s="7" t="s">
         <v>229</v>
-      </c>
-      <c r="O30" s="7" t="s">
-        <v>230</v>
       </c>
       <c r="P30" s="10"/>
     </row>
-    <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="B31" s="7" t="s">
         <v>231</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>232</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>130</v>
+        <v>74</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G31" s="8"/>
+        <v>60</v>
+      </c>
+      <c r="G31" s="8" t="n">
+        <v>9</v>
+      </c>
       <c r="H31" s="8" t="n">
         <v>11</v>
       </c>
@@ -35924,15 +35922,17 @@
         <v>0</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K31" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L31" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="L31" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="M31" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="M31" s="8"/>
       <c r="N31" s="7" t="s">
         <v>234</v>
       </c>
@@ -35974,7 +35974,7 @@
         <v>2</v>
       </c>
       <c r="L32" s="9" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="M32" s="9" t="s">
         <v>238</v>
@@ -36046,7 +36046,7 @@
         <v>35</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>67</v>
@@ -36092,7 +36092,7 @@
         <v>35</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>67</v>
@@ -36121,7 +36121,7 @@
         <v>256</v>
       </c>
       <c r="O35" s="7" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P35" s="10"/>
     </row>
@@ -36278,7 +36278,7 @@
         <v>35</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E39" s="7" t="s">
         <v>67</v>
@@ -36517,7 +36517,7 @@
         <v>36</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>60</v>
@@ -36562,7 +36562,7 @@
         <v>35</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E45" s="7" t="s">
         <v>67</v>
@@ -36611,7 +36611,7 @@
         <v>36</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F46" s="12" t="s">
         <v>60</v>
@@ -36639,7 +36639,7 @@
         <v>320</v>
       </c>
       <c r="O46" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P46" s="10"/>
     </row>
@@ -36685,7 +36685,7 @@
         <v>324</v>
       </c>
       <c r="O47" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P47" s="10"/>
     </row>
@@ -36729,7 +36729,7 @@
         <v>327</v>
       </c>
       <c r="O48" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P48" s="10"/>
     </row>
@@ -36773,7 +36773,7 @@
         <v>331</v>
       </c>
       <c r="O49" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P49" s="10"/>
     </row>
@@ -36788,10 +36788,10 @@
         <v>318</v>
       </c>
       <c r="D50" s="12" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E50" s="12" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="F50" s="12" t="s">
         <v>52</v>
@@ -36817,7 +36817,7 @@
         <v>335</v>
       </c>
       <c r="O50" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P50" s="10"/>
     </row>
@@ -36832,7 +36832,7 @@
         <v>318</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E51" s="12" t="s">
         <v>338</v>
@@ -36861,7 +36861,7 @@
         <v>340</v>
       </c>
       <c r="O51" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P51" s="10"/>
     </row>
@@ -36907,7 +36907,7 @@
         <v>344</v>
       </c>
       <c r="O52" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P52" s="10"/>
     </row>
@@ -36922,10 +36922,10 @@
         <v>318</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E53" s="12" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="F53" s="12" t="s">
         <v>52</v>
@@ -36951,7 +36951,7 @@
         <v>348</v>
       </c>
       <c r="O53" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P53" s="10"/>
     </row>
@@ -36966,10 +36966,10 @@
         <v>318</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E54" s="12" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="F54" s="12" t="s">
         <v>60</v>
@@ -36997,7 +36997,7 @@
         <v>351</v>
       </c>
       <c r="O54" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P54" s="10"/>
     </row>
@@ -37041,7 +37041,7 @@
         <v>355</v>
       </c>
       <c r="O55" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P55" s="10"/>
     </row>
@@ -37087,7 +37087,7 @@
         <v>360</v>
       </c>
       <c r="O56" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P56" s="10"/>
     </row>
@@ -37102,10 +37102,10 @@
         <v>318</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="F57" s="12" t="s">
         <v>52</v>
@@ -37124,14 +37124,14 @@
         <v>3</v>
       </c>
       <c r="L57" s="14" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="M57" s="13"/>
       <c r="N57" s="12" t="s">
         <v>363</v>
       </c>
       <c r="O57" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P57" s="10"/>
     </row>
@@ -37175,7 +37175,7 @@
         <v>367</v>
       </c>
       <c r="O58" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P58" s="10"/>
     </row>
@@ -37193,7 +37193,7 @@
         <v>36</v>
       </c>
       <c r="E59" s="12" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="F59" s="12" t="s">
         <v>60</v>
@@ -37221,7 +37221,7 @@
         <v>371</v>
       </c>
       <c r="O59" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P59" s="10"/>
     </row>
@@ -37239,7 +37239,7 @@
         <v>36</v>
       </c>
       <c r="E60" s="12" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="F60" s="12" t="s">
         <v>52</v>
@@ -37265,7 +37265,7 @@
         <v>375</v>
       </c>
       <c r="O60" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P60" s="10"/>
     </row>
@@ -37283,7 +37283,7 @@
         <v>36</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="F61" s="12" t="s">
         <v>52</v>
@@ -37309,7 +37309,7 @@
         <v>379</v>
       </c>
       <c r="O61" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P61" s="10"/>
     </row>
@@ -37324,7 +37324,7 @@
         <v>318</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E62" s="12" t="s">
         <v>67</v>
@@ -37353,7 +37353,7 @@
         <v>383</v>
       </c>
       <c r="O62" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P62" s="10"/>
     </row>
@@ -37397,7 +37397,7 @@
         <v>387</v>
       </c>
       <c r="O63" s="12" t="s">
-        <v>235</v>
+        <v>152</v>
       </c>
       <c r="P63" s="10"/>
     </row>

</xml_diff>

<commit_message>
beta v0.12.21: rarer cosmetics, compass cooldown 1.5s, boss-fight perfect dodge gives 1 ink
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -17775,7 +17775,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.8 </t>
+      <t xml:space="preserve">1.5 </t>
     </r>
     <r>
       <rPr>
@@ -27894,7 +27894,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">5</t>
+      <t xml:space="preserve">8</t>
     </r>
     <r>
       <rPr>
@@ -27913,7 +27913,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12</t>
+      <t xml:space="preserve">16</t>
     </r>
     <r>
       <rPr>
@@ -27932,7 +27932,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">20</t>
+      <t xml:space="preserve">24</t>
     </r>
   </si>
   <si>
@@ -38552,7 +38552,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>446</v>
@@ -38571,7 +38571,7 @@
       </c>
       <c r="M7" s="7" t="n">
         <f aca="false">ROUND(E7*F7/G7,1)</f>
-        <v>11.1</v>
+        <v>13.3</v>
       </c>
       <c r="N7" s="7" t="s">
         <v>501</v>
@@ -39591,7 +39591,7 @@
         <v>650</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
       <c r="E10" s="10"/>
     </row>
@@ -39606,7 +39606,7 @@
         <v>652</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E11" s="10"/>
     </row>
@@ -39621,7 +39621,7 @@
         <v>652</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E12" s="10"/>
     </row>
@@ -39651,7 +39651,7 @@
         <v>659</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>0.2</v>
+        <v>0.35</v>
       </c>
       <c r="E14" s="10"/>
     </row>

</xml_diff>

<commit_message>
beta v0.12.22: slingshot 65/1.5s/pierce bonus/wall pass/80% guard, depth difficulty, harder achievement tiers, clear seal
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -28670,7 +28670,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">600</t>
+      <t xml:space="preserve">800</t>
     </r>
     <r>
       <rPr>
@@ -28689,7 +28689,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1200</t>
+      <t xml:space="preserve">2000</t>
     </r>
   </si>
   <si>
@@ -28750,8 +28750,457 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">60</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">150</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">首領退散</t>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗第一個首領</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">首領獵人</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計擊敗 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個首領</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">45</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">全員到齊</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗全部 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">種首領</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">瓶安歸來</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗巨型墨瓶 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">40</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">剪單明瞭</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗剪刀魔 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">書途同歸</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗墨跡之書 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">金榜題名</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗考卷魔王 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">妙筆生花</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗巨筆暴君 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">鐘於解脫</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗大鬧鐘 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">精打細算</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗加減法官 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">目中無人</t>
+  </si>
+  <si>
+    <t xml:space="preserve">無傷擊敗一個首領</t>
+  </si>
+  <si>
+    <t xml:space="preserve">無傷大雅</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">無傷清除 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁戰鬥</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -28769,58 +29218,1034 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">45</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">千鈞一髮</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">只剩 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點生命時清除一頁</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">閃亮登場</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">衝刺閃過攻擊 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">150</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">400</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">閃身步</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內成功衝刺閃過攻擊 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">一支穿雲劍</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用穿透筆一發同時穿過 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個敵人</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">易燃易爆炸</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計打破 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個油桶</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">150</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">300</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">箱當然耳</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計打破 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個箱子</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">桶歸於盡</t>
+  </si>
+  <si>
+    <t xml:space="preserve">被油桶炸死一次</t>
+  </si>
+  <si>
+    <t xml:space="preserve">暈籌帷幄</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">移動或瞄準方向連續轉 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">圈（左右搖桿都可以，中間可停一下）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">牌山倒海</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計使用 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">250 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">張卡牌</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">250</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2500</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">合而為一</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">合成升級卡牌 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">90</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">200</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">招搖過市</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計施放 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次特殊卡</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">200</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">450</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">第一頁</t>
+  </si>
+  <si>
+    <t xml:space="preserve">完成第一局冒險（筆記本或課表）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">翻頁不停</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計清除 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁戰鬥</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">寫完了！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">完成整本筆記本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">課不容緩</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式抵達第 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">遊刃有餘</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">贏得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">場事件小遊戲</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">80</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">首領退散</t>
-  </si>
-  <si>
-    <t xml:space="preserve">擊敗第一個首領</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">首領獵人</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計擊敗 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個首領</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6</t>
+    <t xml:space="preserve">買力十足</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">在商店購買 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">小有名氣</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">達到等級 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「十」分完美</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">達到等級 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">墨跡未乾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">用金幣復活一次</t>
+  </si>
+  <si>
+    <t xml:space="preserve">衣見鍾情</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">儲存 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">套自訂套組</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">衣衣不捨</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">收集 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個新顏色或配飾</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
     </r>
     <r>
       <rPr>
@@ -28839,7 +30264,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12</t>
+      <t xml:space="preserve">25</t>
     </r>
     <r>
       <rPr>
@@ -28858,62 +30283,109 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">25</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">全員到齊</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗全部 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">種首領</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">瓶安歸來</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗巨型墨瓶 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
+      <t xml:space="preserve">50</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">文具控</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">種不同武器完成冒險</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">扭轉乾坤</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用遺物扭蛋機抽 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
     </r>
     <r>
       <rPr>
@@ -28933,7 +30405,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">10</t>
+      <t xml:space="preserve">1</t>
     </r>
     <r>
       <rPr>
@@ -28952,7 +30424,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">20</t>
+      <t xml:space="preserve">8</t>
     </r>
     <r>
       <rPr>
@@ -28971,1479 +30443,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">30</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">剪單明瞭</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗剪刀魔 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">書途同歸</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗墨跡之書 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">金榜題名</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗考卷魔王 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">妙筆生花</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗巨筆暴君 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">鐘於解脫</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗大鬧鐘 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">精打細算</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗加減法官 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">目中無人</t>
-  </si>
-  <si>
-    <t xml:space="preserve">無傷擊敗一個首領</t>
-  </si>
-  <si>
-    <t xml:space="preserve">無傷大雅</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">無傷清除 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁戰鬥</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">60</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">千鈞一髮</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">只剩 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">點生命時清除一頁</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">閃亮登場</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">衝刺閃過攻擊 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">80</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">150</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">閃身步</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內成功衝刺閃過攻擊 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">一支穿雲劍</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用穿透筆一發同時穿過 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個敵人</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">易燃易爆炸</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計打破 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個油桶</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">80</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">120</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">箱當然耳</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計打破 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個箱子</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">桶歸於盡</t>
-  </si>
-  <si>
-    <t xml:space="preserve">被油桶炸死一次</t>
-  </si>
-  <si>
-    <t xml:space="preserve">暈籌帷幄</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">移動或瞄準方向連續轉 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">圈（左右搖桿都可以，中間可停一下）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">牌山倒海</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計使用 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">250 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">張卡牌</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">250</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">600</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1200</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">合而為一</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">合成升級卡牌 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">招搖過市</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計施放 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">60 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次特殊卡</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">60</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">120</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">250</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">第一頁</t>
-  </si>
-  <si>
-    <t xml:space="preserve">完成第一局冒險（筆記本或課表）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">翻頁不停</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計清除 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁戰鬥</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">寫完了！</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">完成整本筆記本 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">課不容緩</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">課表模式抵達第 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">遊刃有餘</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">贏得 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">場事件小遊戲</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">買力十足</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">在商店購買 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">小有名氣</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">達到等級 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「十」分完美</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">達到等級 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">墨跡未乾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">用金幣復活一次</t>
-  </si>
-  <si>
-    <t xml:space="preserve">衣見鍾情</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">儲存 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">套自訂套組</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">衣衣不捨</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">收集 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個新顏色或配飾</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">文具控</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">種不同武器完成冒險</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">扭轉乾坤</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用遺物扭蛋機抽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
+      <t xml:space="preserve">15</t>
     </r>
   </si>
   <si>

</xml_diff>

<commit_message>
beta v0.12.23: smoother achievement tier curve
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -28631,7 +28631,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">150 </t>
+      <t xml:space="preserve">250 </t>
     </r>
     <r>
       <rPr>
@@ -28651,7 +28651,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">150</t>
+      <t xml:space="preserve">250</t>
     </r>
     <r>
       <rPr>
@@ -28670,7 +28670,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">800</t>
+      <t xml:space="preserve">700</t>
     </r>
     <r>
       <rPr>
@@ -28689,49 +28689,1011 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">1500</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">精益求精</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計擊倒 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個菁英敵人</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">65</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">130</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">首領退散</t>
+  </si>
+  <si>
+    <t xml:space="preserve">擊敗第一個首領</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">首領獵人</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計擊敗 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個首領</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">35</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">全員到齊</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗全部 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">種首領</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">瓶安歸來</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗巨型墨瓶 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">28</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">剪單明瞭</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗剪刀魔 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">書途同歸</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗墨跡之書 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">金榜題名</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗考卷魔王 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">妙筆生花</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗巨筆暴君 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">鐘於解脫</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗大鬧鐘 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">精打細算</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊敗加減法官 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">目中無人</t>
+  </si>
+  <si>
+    <t xml:space="preserve">無傷擊敗一個首領</t>
+  </si>
+  <si>
+    <t xml:space="preserve">無傷大雅</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">無傷清除 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁戰鬥</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">90</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">千鈞一髮</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">只剩 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點生命時清除一頁</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">閃亮登場</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">衝刺閃過攻擊 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">140</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">300</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">閃身步</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒內成功衝刺閃過攻擊 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">一支穿雲劍</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用穿透筆一發同時穿過 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個敵人</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">易燃易爆炸</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計打破 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個油桶</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">140</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">250</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">箱當然耳</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計打破 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個箱子</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">桶歸於盡</t>
+  </si>
+  <si>
+    <t xml:space="preserve">被油桶炸死一次</t>
+  </si>
+  <si>
+    <t xml:space="preserve">暈籌帷幄</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">移動或瞄準方向連續轉 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">圈（左右搖桿都可以，中間可停一下）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">牌山倒海</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計使用 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">400 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">張卡牌</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">400</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">2000</t>
     </r>
   </si>
   <si>
-    <t xml:space="preserve">精益求精</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計擊倒 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個菁英敵人</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15</t>
+    <t xml:space="preserve">合而為一</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">合成升級卡牌 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">35 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">35</t>
     </r>
     <r>
       <rPr>
@@ -28750,7 +29712,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">60</t>
+      <t xml:space="preserve">80</t>
     </r>
     <r>
       <rPr>
@@ -28769,49 +29731,691 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">150</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">首領退散</t>
-  </si>
-  <si>
-    <t xml:space="preserve">擊敗第一個首領</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">首領獵人</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計擊敗 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個首領</t>
-    </r>
-  </si>
-  <si>
+      <t xml:space="preserve">160</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">招搖過市</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計施放 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">90 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次特殊卡</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">90</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">200</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">380</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">第一頁</t>
+  </si>
+  <si>
+    <t xml:space="preserve">完成第一局冒險（筆記本或課表）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">翻頁不停</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">累計清除 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">60 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁戰鬥</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">寫完了！</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">完成整本筆記本 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">課不容緩</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">課表模式抵達第 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頁</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">遊刃有餘</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">贏得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">場事件小遊戲</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">70</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">買力十足</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">在商店購買 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">小有名氣</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">達到等級 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">「十」分完美</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">達到等級 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">墨跡未乾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">用金幣復活一次</t>
+  </si>
+  <si>
+    <t xml:space="preserve">衣見鍾情</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">儲存 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">套自訂套組</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">衣衣不捨</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">收集 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個新顏色或配飾</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">25</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">文具控</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">種不同武器完成冒險</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">扭轉乾坤</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用遺物扭蛋機抽 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -28839,1611 +30443,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">45</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">全員到齊</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗全部 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">種首領</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">瓶安歸來</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗巨型墨瓶 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">剪單明瞭</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗剪刀魔 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">書途同歸</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗墨跡之書 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">金榜題名</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗考卷魔王 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">妙筆生花</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗巨筆暴君 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">鐘於解脫</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗大鬧鐘 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">精打細算</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">擊敗加減法官 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">目中無人</t>
-  </si>
-  <si>
-    <t xml:space="preserve">無傷擊敗一個首領</t>
-  </si>
-  <si>
-    <t xml:space="preserve">無傷大雅</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">無傷清除 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁戰鬥</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
       <t xml:space="preserve">12</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">45</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">100</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">千鈞一髮</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">只剩 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">點生命時清除一頁</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">閃亮登場</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">衝刺閃過攻擊 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">150</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">400</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">閃身步</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">秒內成功衝刺閃過攻擊 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">一支穿雲劍</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用穿透筆一發同時穿過 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個敵人</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">易燃易爆炸</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計打破 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個油桶</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">150</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">300</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">箱當然耳</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計打破 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個箱子</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">桶歸於盡</t>
-  </si>
-  <si>
-    <t xml:space="preserve">被油桶炸死一次</t>
-  </si>
-  <si>
-    <t xml:space="preserve">暈籌帷幄</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">移動或瞄準方向連續轉 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">圈（左右搖桿都可以，中間可停一下）</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">牌山倒海</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計使用 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">250 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">張卡牌</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">250</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1000</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2500</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">合而為一</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">合成升級卡牌 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">90</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">200</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">招搖過市</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計施放 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">60 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次特殊卡</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">60</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">200</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">450</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">第一頁</t>
-  </si>
-  <si>
-    <t xml:space="preserve">完成第一局冒險（筆記本或課表）</t>
-  </si>
-  <si>
-    <t xml:space="preserve">翻頁不停</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">累計清除 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁戰鬥</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">寫完了！</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">完成整本筆記本 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">課不容緩</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">課表模式抵達第 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">頁</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">30</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">遊刃有餘</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">贏得 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">場事件小遊戲</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">40</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">80</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">買力十足</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">在商店購買 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">小有名氣</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">達到等級 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">「十」分完美</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">達到等級 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">墨跡未乾</t>
-  </si>
-  <si>
-    <t xml:space="preserve">用金幣復活一次</t>
-  </si>
-  <si>
-    <t xml:space="preserve">衣見鍾情</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">儲存 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">套自訂套組</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">衣衣不捨</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">收集 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">個新顏色或配飾</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">25</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">文具控</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">種不同武器完成冒險</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">扭轉乾坤</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">用遺物扭蛋機抽 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">次</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">／</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">15</t>
     </r>
   </si>
   <si>

</xml_diff>

<commit_message>
beta v0.12.25: compensate only pre-change slingshot owners, clear achievement 1/5/10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -29908,7 +29908,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">3</t>
+      <t xml:space="preserve">5</t>
     </r>
     <r>
       <rPr>
@@ -29927,7 +29927,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">7</t>
+      <t xml:space="preserve">10</t>
     </r>
   </si>
   <si>

</xml_diff>

<commit_message>
beta v0.12.28: six new relics (spare hand, red pen, pedometer, four-leaf clover, cheat sheet, clipboard)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1316" uniqueCount="905">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1333" uniqueCount="921">
   <si>
     <r>
       <rPr>
@@ -32326,6 +32326,326 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">0.5</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">備用手牌</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">每頁的重抽次數 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（可與「備用彈匣」增加的次數累積）；頭目連戰中每場頭目戰算一頁。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">redraw</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">紅筆批改</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">對菁英與頭目造成的傷害 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+10%</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">，對一般敵人無效。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">倍率：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.1</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">計步器</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">有戰鬥的頁面全程沒有扣血時，戰鬥結束回復 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點墨水（不超過上限）。紙盾、金光護盾等擋下的傷害不算受傷；商店、休息區、事件等沒有戰鬥的頁面不會觸發。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">墨水：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">幸運草</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">擊倒敵人時有 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4% </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">機率回復 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">點生命，每頁最多 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次（生命全滿時不會觸發）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">chance</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.04
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">回復：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">上限：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">小抄</t>
+  </si>
+  <si>
+    <t xml:space="preserve">每頁打出的第一張一般牌不消耗墨水（特殊技不算）；頭目連戰中每場頭目戰各算一次。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">墊板</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">頭目戰開場時墨水回滿，並獲得 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">片沒有時間限制的紙盾，會一直留到擋下一次傷害為止（和其他紙盾分開計算，總數不超過紙盾上限）。</t>
     </r>
   </si>
   <si>
@@ -40563,7 +40883,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -40961,11 +41281,105 @@
         <v>869</v>
       </c>
       <c r="C24" s="7"/>
-      <c r="D24" s="7" t="n">
+      <c r="D24" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="E24" s="7"/>
+      <c r="E24" s="6" t="s">
+        <v>870</v>
+      </c>
       <c r="F24" s="10"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="7" t="s">
+        <v>871</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>872</v>
+      </c>
+      <c r="C25" s="7"/>
+      <c r="D25" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>873</v>
+      </c>
+      <c r="F25" s="10"/>
+    </row>
+    <row r="26" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
+        <v>874</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>875</v>
+      </c>
+      <c r="C26" s="7"/>
+      <c r="D26" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>876</v>
+      </c>
+      <c r="F26" s="10"/>
+    </row>
+    <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="7" t="s">
+        <v>877</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>878</v>
+      </c>
+      <c r="C27" s="7"/>
+      <c r="D27" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>879</v>
+      </c>
+      <c r="F27" s="10"/>
+    </row>
+    <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="7" t="s">
+        <v>880</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>881</v>
+      </c>
+      <c r="C28" s="7"/>
+      <c r="D28" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E28" s="7"/>
+      <c r="F28" s="10"/>
+    </row>
+    <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="7" t="s">
+        <v>882</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>883</v>
+      </c>
+      <c r="C29" s="7"/>
+      <c r="D29" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>858</v>
+      </c>
+      <c r="F29" s="10"/>
+    </row>
+    <row r="30" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="7" t="s">
+        <v>884</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>885</v>
+      </c>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="E30" s="7"/>
+      <c r="F30" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -40997,7 +41411,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>870</v>
+        <v>886</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>628</v>
@@ -41006,10 +41420,10 @@
         <v>480</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>871</v>
+        <v>887</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>872</v>
+        <v>888</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>802</v>
@@ -41020,115 +41434,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>873</v>
+        <v>889</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>874</v>
+        <v>890</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>875</v>
+        <v>891</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>876</v>
+        <v>892</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>877</v>
+        <v>893</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>878</v>
+        <v>894</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>879</v>
+        <v>895</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>880</v>
+        <v>896</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>881</v>
+        <v>897</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>882</v>
+        <v>898</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>883</v>
+        <v>899</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>884</v>
+        <v>900</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>885</v>
+        <v>901</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>886</v>
+        <v>902</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>887</v>
+        <v>903</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>888</v>
+        <v>904</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>889</v>
+        <v>905</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>890</v>
+        <v>906</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>891</v>
+        <v>907</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>892</v>
+        <v>908</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>893</v>
+        <v>909</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>894</v>
+        <v>910</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>895</v>
+        <v>911</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>896</v>
+        <v>912</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>897</v>
+        <v>913</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>898</v>
+        <v>914</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>899</v>
+        <v>915</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>900</v>
+        <v>916</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>901</v>
+        <v>917</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>902</v>
+        <v>918</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>903</v>
+        <v>919</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>904</v>
+        <v>920</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
beta v0.12.29: new enemies paper pilot (S-curve paper plane) and sticky note helper (paper shields)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1333" uniqueCount="921">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1343" uniqueCount="929">
   <si>
     <r>
       <rPr>
@@ -14186,6 +14186,496 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">paperPlane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">紙飛機兵</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">S </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">形紙飛機】地面先出現 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">S </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">形虛線，紙飛機飛到你身後再沿反向 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">S </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">形飛回，去回各打 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">次；會飛越矮牆，被打中就墜毀並讓紙飛機兵硬直。
+【雙機交叉（精英）】一次擲出兩架，一左一右在途中交叉，回程也交叉；預警縮短為 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒，兩架都被打掉才硬直。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">range</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[6, 10]
+strafe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.7
+firstThrow</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[1.6, 2.4]
+throwEvery</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[1.6, 2.2]
+telegraph</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6
+eliteTelegraph</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5
+lead</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2
+flyRange</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[8, 13]
+amp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.2
+outSpeed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8
+backSpeed</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">9.5
+hover</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.35
+planeRadius</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.45
+planeHeight</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.2
+planeDamage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1
+rehit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.5
+stagger</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.6
+throwSlow</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.4
+dashes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">22
+dashAlpha</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.4
+maxAlive</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">bird</t>
   </si>
   <si>
@@ -14364,6 +14854,228 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">1</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">stickyHelper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">便利貼助手</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【貼紙盾】每 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒替最近、沒有盾的敵人貼便利貼：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">以下的一擊完全擋下，更強的扣 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">後打穿；助手倒下時全部消失。
+【孤軍衝鋒】場上只剩它（或只剩便利貼助手）時，會直接衝向你用身體撞擊。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">keep</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8
+behind</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2.6
+stickEvery</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4
+blockMax</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20
+pierceLoss</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10
+rush</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1.35
+noteSize</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.55
+maxAlive</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
     </r>
   </si>
   <si>
@@ -37739,7 +38451,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -38060,7 +38772,7 @@
       </c>
       <c r="P8" s="10"/>
     </row>
-    <row r="9" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="283.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
         <v>426</v>
       </c>
@@ -38068,17 +38780,17 @@
         <v>427</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>423</v>
+        <v>404</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="E9" s="7" t="n">
         <f aca="false">ROUND(D9*$B$1,0)</f>
-        <v>65</v>
+        <v>100</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>6.5</v>
+        <v>2.4</v>
       </c>
       <c r="G9" s="8" t="n">
         <v>1</v>
@@ -38087,14 +38799,14 @@
       <c r="I9" s="8"/>
       <c r="J9" s="8"/>
       <c r="K9" s="8" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="L9" s="7" t="n">
         <f aca="false">K9*$D$1</f>
+        <v>3</v>
+      </c>
+      <c r="M9" s="8" t="n">
         <v>2</v>
-      </c>
-      <c r="M9" s="8" t="n">
-        <v>1</v>
       </c>
       <c r="N9" s="7" t="s">
         <v>428</v>
@@ -38104,7 +38816,7 @@
       </c>
       <c r="P9" s="10"/>
     </row>
-    <row r="10" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
         <v>430</v>
       </c>
@@ -38112,30 +38824,24 @@
         <v>431</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>404</v>
+        <v>423</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>58</v>
+        <v>26</v>
       </c>
       <c r="E10" s="7" t="n">
         <f aca="false">ROUND(D10*$B$1,0)</f>
-        <v>145</v>
+        <v>65</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>2.2</v>
+        <v>6.5</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>432</v>
-      </c>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
       <c r="K10" s="8" t="n">
         <v>1</v>
       </c>
@@ -38144,35 +38850,35 @@
         <v>2</v>
       </c>
       <c r="M10" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N10" s="7" t="s">
+        <v>432</v>
+      </c>
+      <c r="O10" s="6" t="s">
         <v>433</v>
-      </c>
-      <c r="O10" s="6" t="s">
-        <v>434</v>
       </c>
       <c r="P10" s="10"/>
     </row>
-    <row r="11" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
+        <v>434</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>435</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>436</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>404</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>90</v>
+        <v>36</v>
       </c>
       <c r="E11" s="7" t="n">
         <f aca="false">ROUND(D11*$B$1,0)</f>
-        <v>225</v>
+        <v>90</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>1</v>
@@ -38181,171 +38887,177 @@
       <c r="I11" s="8"/>
       <c r="J11" s="8"/>
       <c r="K11" s="8" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="L11" s="7" t="n">
         <f aca="false">K11*$D$1</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M11" s="8" t="n">
         <v>2</v>
       </c>
       <c r="N11" s="7" t="s">
+        <v>436</v>
+      </c>
+      <c r="O11" s="6" t="s">
         <v>437</v>
-      </c>
-      <c r="O11" s="6" t="s">
-        <v>438</v>
       </c>
       <c r="P11" s="10"/>
     </row>
-    <row r="12" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>439</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>409</v>
-      </c>
       <c r="C12" s="7" t="s">
-        <v>440</v>
+        <v>404</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">ROUND(D12*$B$1,0)</f>
-        <v>35</v>
+        <v>145</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>4.2</v>
+        <v>2.2</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
+      <c r="H12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>440</v>
+      </c>
       <c r="K12" s="8" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L12" s="7" t="n">
         <f aca="false">K12*$D$1</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M12" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N12" s="7"/>
+        <v>2</v>
+      </c>
+      <c r="N12" s="7" t="s">
+        <v>441</v>
+      </c>
       <c r="O12" s="6" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="P12" s="10"/>
     </row>
-    <row r="13" customFormat="false" ht="228.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>442</v>
-      </c>
-      <c r="B13" s="12" t="s">
+    <row r="13" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>443</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="B13" s="7" t="s">
         <v>444</v>
       </c>
-      <c r="D13" s="13" t="n">
-        <v>900</v>
-      </c>
-      <c r="E13" s="12" t="s">
+      <c r="C13" s="7" t="s">
+        <v>404</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <f aca="false">ROUND(D13*$B$1,0)</f>
+        <v>225</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <f aca="false">K13*$D$1</f>
+        <v>3</v>
+      </c>
+      <c r="M13" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" s="7" t="s">
         <v>445</v>
       </c>
-      <c r="F13" s="13" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G13" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="J13" s="13"/>
-      <c r="K13" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" s="11" t="s">
+      <c r="O13" s="6" t="s">
         <v>446</v>
-      </c>
-      <c r="M13" s="13"/>
-      <c r="N13" s="12" t="s">
-        <v>447</v>
-      </c>
-      <c r="O13" s="11" t="s">
-        <v>448</v>
       </c>
       <c r="P13" s="10"/>
     </row>
-    <row r="14" customFormat="false" ht="174.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="s">
+    <row r="14" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <f aca="false">ROUND(D14*$B$1,0)</f>
+        <v>35</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <f aca="false">K14*$D$1</f>
+        <v>1</v>
+      </c>
+      <c r="M14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" s="7"/>
+      <c r="O14" s="6" t="s">
         <v>449</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>450</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>444</v>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>445</v>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="G14" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="L14" s="11" t="s">
-        <v>446</v>
-      </c>
-      <c r="M14" s="13"/>
-      <c r="N14" s="12" t="s">
-        <v>451</v>
-      </c>
-      <c r="O14" s="11" t="s">
-        <v>452</v>
       </c>
       <c r="P14" s="10"/>
     </row>
-    <row r="15" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="228.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
+        <v>450</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>451</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>452</v>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>900</v>
+      </c>
+      <c r="E15" s="12" t="s">
         <v>453</v>
       </c>
-      <c r="B15" s="12" t="s">
-        <v>454</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>444</v>
-      </c>
-      <c r="D15" s="13" t="n">
-        <v>1300</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>445</v>
-      </c>
       <c r="F15" s="13" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="G15" s="13" t="n">
         <v>1</v>
@@ -38354,14 +39066,14 @@
         <v>1</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="J15" s="13"/>
       <c r="K15" s="13" t="n">
         <v>4</v>
       </c>
       <c r="L15" s="11" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="M15" s="13"/>
       <c r="N15" s="12" t="s">
@@ -38372,7 +39084,7 @@
       </c>
       <c r="P15" s="10"/>
     </row>
-    <row r="16" customFormat="false" ht="331.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="174.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
         <v>457</v>
       </c>
@@ -38380,16 +39092,16 @@
         <v>458</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="G16" s="13" t="n">
         <v>1</v>
@@ -38398,14 +39110,14 @@
         <v>1</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J16" s="13"/>
       <c r="K16" s="13" t="n">
         <v>4</v>
       </c>
       <c r="L16" s="11" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="12" t="s">
@@ -38416,7 +39128,7 @@
       </c>
       <c r="P16" s="10"/>
     </row>
-    <row r="17" customFormat="false" ht="252.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
         <v>461</v>
       </c>
@@ -38424,13 +39136,13 @@
         <v>462</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>1300</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="F17" s="13" t="n">
         <v>0</v>
@@ -38442,14 +39154,14 @@
         <v>1</v>
       </c>
       <c r="I17" s="13" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="J17" s="13"/>
       <c r="K17" s="13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L17" s="11" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="M17" s="13"/>
       <c r="N17" s="12" t="s">
@@ -38460,7 +39172,7 @@
       </c>
       <c r="P17" s="10"/>
     </row>
-    <row r="18" customFormat="false" ht="381.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="331.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
         <v>465</v>
       </c>
@@ -38468,16 +39180,16 @@
         <v>466</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>1300</v>
+        <v>1100</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>1</v>
@@ -38485,13 +39197,15 @@
       <c r="H18" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="13"/>
+      <c r="I18" s="13" t="n">
+        <v>7</v>
+      </c>
       <c r="J18" s="13"/>
       <c r="K18" s="13" t="n">
         <v>4</v>
       </c>
       <c r="L18" s="11" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="M18" s="13"/>
       <c r="N18" s="12" t="s">
@@ -38502,47 +39216,133 @@
       </c>
       <c r="P18" s="10"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+    <row r="19" customFormat="false" ht="252.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
         <v>469</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="12" t="s">
         <v>470</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="12" t="s">
+        <v>452</v>
+      </c>
+      <c r="D19" s="13" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>453</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="L19" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="M19" s="13"/>
+      <c r="N19" s="12" t="s">
+        <v>471</v>
+      </c>
+      <c r="O19" s="11" t="s">
+        <v>472</v>
+      </c>
+      <c r="P19" s="10"/>
+    </row>
+    <row r="20" customFormat="false" ht="381.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
+        <v>473</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>474</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>452</v>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>453</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="L20" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="M20" s="13"/>
+      <c r="N20" s="12" t="s">
+        <v>475</v>
+      </c>
+      <c r="O20" s="11" t="s">
+        <v>476</v>
+      </c>
+      <c r="P20" s="10"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>404</v>
       </c>
-      <c r="D19" s="8" t="n">
+      <c r="D21" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="E19" s="7" t="n">
-        <f aca="false">ROUND(D19*$B$1,0)</f>
+      <c r="E21" s="7" t="n">
+        <f aca="false">ROUND(D21*$B$1,0)</f>
         <v>113</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="F21" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="8" t="n">
+      <c r="G21" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8" t="n">
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="L19" s="7" t="n">
-        <f aca="false">K19*$D$1</f>
+      <c r="L21" s="7" t="n">
+        <f aca="false">K21*$D$1</f>
         <v>1</v>
       </c>
-      <c r="M19" s="8" t="n">
+      <c r="M21" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N19" s="7"/>
-      <c r="O19" s="6" t="s">
-        <v>471</v>
-      </c>
-      <c r="P19" s="10"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="P21" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -38590,37 +39390,37 @@
         <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>472</v>
+        <v>480</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>473</v>
+        <v>481</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>396</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>475</v>
+        <v>483</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>476</v>
+        <v>484</v>
       </c>
       <c r="J1" s="5" t="s">
         <v>395</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>478</v>
+        <v>486</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>479</v>
+        <v>487</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>480</v>
+        <v>488</v>
       </c>
       <c r="O1" s="5" t="s">
         <v>32</v>
@@ -38628,16 +39428,16 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>481</v>
+        <v>489</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>482</v>
+        <v>490</v>
       </c>
       <c r="C2" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>483</v>
+        <v>491</v>
       </c>
       <c r="E2" s="8" t="n">
         <v>10</v>
@@ -38672,16 +39472,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>484</v>
+        <v>492</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>485</v>
+        <v>493</v>
       </c>
       <c r="C3" s="8" t="n">
         <v>3</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>486</v>
+        <v>494</v>
       </c>
       <c r="E3" s="8" t="n">
         <v>5</v>
@@ -38716,16 +39516,16 @@
     </row>
     <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>487</v>
+        <v>495</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>488</v>
+        <v>496</v>
       </c>
       <c r="C4" s="8" t="n">
         <v>5</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>489</v>
+        <v>497</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>15</v>
@@ -38756,22 +39556,22 @@
         <v>24.2</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>490</v>
+        <v>498</v>
       </c>
       <c r="O4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>491</v>
+        <v>499</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>492</v>
+        <v>500</v>
       </c>
       <c r="C5" s="8" t="n">
         <v>7</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>493</v>
+        <v>501</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>12</v>
@@ -38802,22 +39602,22 @@
         <v>72</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>494</v>
+        <v>502</v>
       </c>
       <c r="O5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>495</v>
+        <v>503</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>496</v>
+        <v>504</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>9</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>497</v>
+        <v>505</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>5</v>
@@ -38835,10 +39635,10 @@
         <v>3</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>0</v>
@@ -38848,22 +39648,22 @@
         <v>50</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>498</v>
+        <v>506</v>
       </c>
       <c r="O6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>499</v>
+        <v>507</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>12</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>500</v>
+        <v>508</v>
       </c>
       <c r="E7" s="8" t="n">
         <v>20</v>
@@ -38875,10 +39675,10 @@
         <v>1.5</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="J7" s="8" t="n">
         <v>20</v>
@@ -38894,22 +39694,22 @@
         <v>13.3</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>501</v>
+        <v>509</v>
       </c>
       <c r="O7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>502</v>
+        <v>510</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>503</v>
+        <v>511</v>
       </c>
       <c r="C8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>504</v>
+        <v>512</v>
       </c>
       <c r="E8" s="8" t="n">
         <v>5</v>
@@ -38940,22 +39740,22 @@
         <v>33.3</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>505</v>
+        <v>513</v>
       </c>
       <c r="O8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>506</v>
+        <v>514</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>507</v>
+        <v>515</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>18</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>508</v>
+        <v>516</v>
       </c>
       <c r="E9" s="8" t="n">
         <v>15</v>
@@ -39016,19 +39816,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>509</v>
+        <v>517</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>510</v>
+        <v>518</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>511</v>
+        <v>519</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>512</v>
+        <v>520</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -39036,325 +39836,325 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>513</v>
+        <v>521</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>515</v>
+        <v>523</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>516</v>
+        <v>524</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>518</v>
+        <v>526</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>519</v>
+        <v>527</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>522</v>
+        <v>530</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>523</v>
+        <v>531</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>524</v>
+        <v>532</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>525</v>
+        <v>533</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>526</v>
+        <v>534</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>527</v>
+        <v>535</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>528</v>
+        <v>536</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>529</v>
+        <v>537</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>82</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>530</v>
+        <v>538</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>531</v>
+        <v>539</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>532</v>
+        <v>540</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>533</v>
+        <v>541</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>534</v>
+        <v>542</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>535</v>
+        <v>543</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>536</v>
+        <v>544</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>537</v>
+        <v>545</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>538</v>
+        <v>546</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>539</v>
+        <v>547</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>540</v>
+        <v>548</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>541</v>
+        <v>549</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>542</v>
+        <v>550</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>543</v>
+        <v>551</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>544</v>
+        <v>552</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>545</v>
+        <v>553</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>546</v>
+        <v>554</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>547</v>
+        <v>555</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>548</v>
+        <v>556</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>549</v>
+        <v>557</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>550</v>
+        <v>558</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>551</v>
+        <v>559</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="216.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>552</v>
+        <v>560</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>553</v>
+        <v>561</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>554</v>
+        <v>562</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>555</v>
+        <v>563</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>556</v>
+        <v>564</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>557</v>
+        <v>565</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>558</v>
+        <v>566</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>559</v>
+        <v>567</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>560</v>
+        <v>568</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>561</v>
+        <v>569</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>562</v>
+        <v>570</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>563</v>
+        <v>571</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>563</v>
+        <v>571</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>564</v>
+        <v>572</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>565</v>
+        <v>573</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>566</v>
+        <v>574</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>569</v>
+        <v>577</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>570</v>
+        <v>578</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>571</v>
+        <v>579</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>572</v>
+        <v>580</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>573</v>
+        <v>581</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>574</v>
+        <v>582</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>575</v>
+        <v>583</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>576</v>
+        <v>584</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>577</v>
+        <v>585</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>578</v>
+        <v>586</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>579</v>
+        <v>587</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>580</v>
+        <v>588</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>581</v>
+        <v>589</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>582</v>
+        <v>590</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>583</v>
+        <v>591</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>584</v>
+        <v>592</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>585</v>
+        <v>593</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>586</v>
+        <v>594</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>587</v>
+        <v>595</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>588</v>
+        <v>596</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>589</v>
+        <v>597</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>590</v>
+        <v>598</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="377.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>591</v>
+        <v>599</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>592</v>
+        <v>600</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>593</v>
+        <v>601</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>594</v>
+        <v>602</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>595</v>
+        <v>603</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>596</v>
+        <v>604</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>597</v>
+        <v>605</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>598</v>
+        <v>606</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>600</v>
+        <v>608</v>
       </c>
       <c r="F19" s="10"/>
     </row>
@@ -39389,13 +40189,13 @@
         <v>20</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>601</v>
+        <v>609</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>602</v>
+        <v>610</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>603</v>
+        <v>611</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -39403,13 +40203,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>605</v>
+        <v>613</v>
       </c>
       <c r="D2" s="16" t="n">
         <f aca="false">ROUND(B2/SUM(B$2:B$13),3)</f>
@@ -39419,13 +40219,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>606</v>
+        <v>614</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">ROUND(B3/SUM(B$2:B$13),3)</f>
@@ -39435,13 +40235,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>607</v>
+        <v>615</v>
       </c>
       <c r="D4" s="16" t="n">
         <f aca="false">ROUND(B4/SUM(B$2:B$13),3)</f>
@@ -39451,13 +40251,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>608</v>
+        <v>616</v>
       </c>
       <c r="D5" s="16" t="n">
         <f aca="false">ROUND(B5/SUM(B$2:B$13),3)</f>
@@ -39467,13 +40267,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>609</v>
+        <v>617</v>
       </c>
       <c r="D6" s="16" t="n">
         <f aca="false">ROUND(B6/SUM(B$2:B$13),3)</f>
@@ -39483,13 +40283,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>610</v>
+        <v>618</v>
       </c>
       <c r="D7" s="16" t="n">
         <f aca="false">ROUND(B7/SUM(B$2:B$13),3)</f>
@@ -39499,13 +40299,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>611</v>
+        <v>619</v>
       </c>
       <c r="D8" s="16" t="n">
         <f aca="false">ROUND(B8/SUM(B$2:B$13),3)</f>
@@ -39515,13 +40315,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>612</v>
+        <v>620</v>
       </c>
       <c r="D9" s="16" t="n">
         <f aca="false">ROUND(B9/SUM(B$2:B$13),3)</f>
@@ -39531,13 +40331,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>613</v>
+        <v>621</v>
       </c>
       <c r="D10" s="16" t="n">
         <f aca="false">ROUND(B10/SUM(B$2:B$13),3)</f>
@@ -39547,13 +40347,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>614</v>
+        <v>622</v>
       </c>
       <c r="D11" s="16" t="n">
         <f aca="false">ROUND(B11/SUM(B$2:B$13),3)</f>
@@ -39563,13 +40363,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>615</v>
+        <v>623</v>
       </c>
       <c r="D12" s="16" t="n">
         <f aca="false">ROUND(B12/SUM(B$2:B$13),3)</f>
@@ -39579,13 +40379,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>604</v>
+        <v>612</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>616</v>
+        <v>624</v>
       </c>
       <c r="D13" s="16" t="n">
         <f aca="false">ROUND(B13/SUM(B$2:B$13),3)</f>
@@ -39595,13 +40395,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>618</v>
+        <v>626</v>
       </c>
       <c r="D14" s="16" t="n">
         <f aca="false">ROUND(B14/SUM(B$14:B$22),3)</f>
@@ -39611,13 +40411,13 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>619</v>
+        <v>627</v>
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">ROUND(B15/SUM(B$14:B$22),3)</f>
@@ -39627,13 +40427,13 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>620</v>
+        <v>628</v>
       </c>
       <c r="D16" s="16" t="n">
         <f aca="false">ROUND(B16/SUM(B$14:B$22),3)</f>
@@ -39643,13 +40443,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>621</v>
+        <v>629</v>
       </c>
       <c r="D17" s="16" t="n">
         <f aca="false">ROUND(B17/SUM(B$14:B$22),3)</f>
@@ -39659,13 +40459,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>622</v>
+        <v>630</v>
       </c>
       <c r="D18" s="16" t="n">
         <f aca="false">ROUND(B18/SUM(B$14:B$22),3)</f>
@@ -39675,13 +40475,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>623</v>
+        <v>631</v>
       </c>
       <c r="D19" s="16" t="n">
         <f aca="false">ROUND(B19/SUM(B$14:B$22),3)</f>
@@ -39691,13 +40491,13 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>624</v>
+        <v>632</v>
       </c>
       <c r="D20" s="16" t="n">
         <f aca="false">ROUND(B20/SUM(B$14:B$22),3)</f>
@@ -39707,13 +40507,13 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="B21" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>625</v>
+        <v>633</v>
       </c>
       <c r="D21" s="16" t="n">
         <f aca="false">ROUND(B21/SUM(B$14:B$22),3)</f>
@@ -39723,13 +40523,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>617</v>
+        <v>625</v>
       </c>
       <c r="B22" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>626</v>
+        <v>634</v>
       </c>
       <c r="D22" s="16" t="n">
         <f aca="false">ROUND(B22/SUM(B$14:B$22),3)</f>
@@ -39765,16 +40565,16 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>627</v>
+        <v>635</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>628</v>
+        <v>636</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>629</v>
+        <v>637</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>32</v>
@@ -39782,13 +40582,13 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>630</v>
+        <v>638</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>631</v>
+        <v>639</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>632</v>
+        <v>640</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>2</v>
@@ -39797,13 +40597,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>630</v>
+        <v>638</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>633</v>
+        <v>641</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>634</v>
+        <v>642</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>5</v>
@@ -39812,13 +40612,13 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>630</v>
+        <v>638</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>635</v>
+        <v>643</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>636</v>
+        <v>644</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>25</v>
@@ -39827,13 +40627,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>637</v>
+        <v>645</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>638</v>
+        <v>646</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>639</v>
+        <v>647</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>1</v>
@@ -39842,13 +40642,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>637</v>
+        <v>645</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>640</v>
+        <v>648</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>641</v>
+        <v>649</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>10</v>
@@ -39857,13 +40657,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>637</v>
+        <v>645</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>642</v>
+        <v>650</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>643</v>
+        <v>651</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2.5</v>
@@ -39872,13 +40672,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>645</v>
+        <v>653</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>646</v>
+        <v>654</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>5</v>
@@ -39887,13 +40687,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>647</v>
+        <v>655</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>648</v>
+        <v>656</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>2</v>
@@ -39902,13 +40702,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>649</v>
+        <v>657</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>650</v>
+        <v>658</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>0.25</v>
@@ -39917,13 +40717,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>651</v>
+        <v>659</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>10</v>
@@ -39932,13 +40732,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>653</v>
+        <v>661</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>652</v>
+        <v>660</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>2</v>
@@ -39947,28 +40747,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>654</v>
+        <v>662</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>655</v>
+        <v>663</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>656</v>
+        <v>664</v>
       </c>
       <c r="E13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>657</v>
+        <v>665</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>658</v>
+        <v>666</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>659</v>
+        <v>667</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>0.35</v>
@@ -39977,28 +40777,28 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>657</v>
+        <v>665</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>660</v>
+        <v>668</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>661</v>
+        <v>669</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>662</v>
+        <v>670</v>
       </c>
       <c r="E15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>644</v>
+        <v>652</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>663</v>
+        <v>671</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>1</v>
@@ -40007,10 +40807,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
@@ -40020,13 +40820,13 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>667</v>
+        <v>675</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>668</v>
+        <v>676</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>5</v>
@@ -40035,10 +40835,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>669</v>
+        <v>677</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
@@ -40048,10 +40848,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>670</v>
+        <v>678</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
@@ -40061,10 +40861,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>671</v>
+        <v>679</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
@@ -40074,13 +40874,13 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>673</v>
+        <v>681</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>674</v>
+        <v>682</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>60000</v>
@@ -40089,13 +40889,13 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>675</v>
+        <v>683</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="D23" s="8" t="n">
         <v>45000</v>
@@ -40104,13 +40904,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>677</v>
+        <v>685</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>35000</v>
@@ -40119,13 +40919,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>679</v>
+        <v>687</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>680</v>
+        <v>688</v>
       </c>
       <c r="D25" s="8" t="n">
         <v>20000</v>
@@ -40134,13 +40934,13 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>681</v>
+        <v>689</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>10000</v>
@@ -40149,13 +40949,13 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>683</v>
+        <v>691</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>684</v>
+        <v>692</v>
       </c>
       <c r="D27" s="8" t="n">
         <v>5000</v>
@@ -40164,13 +40964,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>674</v>
+        <v>682</v>
       </c>
       <c r="D28" s="8" t="n">
         <v>60000</v>
@@ -40179,13 +40979,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>686</v>
+        <v>694</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>676</v>
+        <v>684</v>
       </c>
       <c r="D29" s="8" t="n">
         <v>45000</v>
@@ -40194,13 +40994,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>678</v>
+        <v>686</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>35000</v>
@@ -40209,13 +41009,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B31" s="7" t="s">
+        <v>696</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>688</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>680</v>
       </c>
       <c r="D31" s="8" t="n">
         <v>20000</v>
@@ -40224,13 +41024,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>689</v>
+        <v>697</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>682</v>
+        <v>690</v>
       </c>
       <c r="D32" s="8" t="n">
         <v>10000</v>
@@ -40239,13 +41039,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>672</v>
+        <v>680</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>690</v>
+        <v>698</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>684</v>
+        <v>692</v>
       </c>
       <c r="D33" s="8" t="n">
         <v>5000</v>
@@ -40254,616 +41054,616 @@
     </row>
     <row r="34" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>692</v>
+        <v>700</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>693</v>
+        <v>701</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>694</v>
+        <v>702</v>
       </c>
       <c r="E34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>695</v>
+        <v>703</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>696</v>
+        <v>704</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>697</v>
+        <v>705</v>
       </c>
       <c r="E35" s="10"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>698</v>
+        <v>706</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>699</v>
+        <v>707</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="E36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>701</v>
+        <v>709</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>702</v>
+        <v>710</v>
       </c>
       <c r="D37" s="8" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
       <c r="E37" s="10"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>704</v>
+        <v>712</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>705</v>
+        <v>713</v>
       </c>
       <c r="D38" s="8" t="s">
-        <v>706</v>
+        <v>714</v>
       </c>
       <c r="E38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>707</v>
+        <v>715</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="E39" s="10"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>710</v>
+        <v>718</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>711</v>
+        <v>719</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="E40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>712</v>
+        <v>720</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>713</v>
+        <v>721</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>714</v>
+        <v>722</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>715</v>
+        <v>723</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="E42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>716</v>
+        <v>724</v>
       </c>
       <c r="C43" s="7" t="s">
+        <v>725</v>
+      </c>
+      <c r="D43" s="8" t="s">
         <v>717</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>709</v>
       </c>
       <c r="E43" s="10"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>718</v>
+        <v>726</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>719</v>
+        <v>727</v>
       </c>
       <c r="D44" s="8" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="E44" s="10"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>720</v>
+        <v>728</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>721</v>
+        <v>729</v>
       </c>
       <c r="D45" s="8" t="s">
-        <v>709</v>
+        <v>717</v>
       </c>
       <c r="E45" s="10"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>722</v>
+        <v>730</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>723</v>
+        <v>731</v>
       </c>
       <c r="D46" s="8" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="E46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>724</v>
+        <v>732</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>725</v>
+        <v>733</v>
       </c>
       <c r="D47" s="8" t="s">
-        <v>726</v>
+        <v>734</v>
       </c>
       <c r="E47" s="10"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>727</v>
+        <v>735</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>728</v>
+        <v>736</v>
       </c>
       <c r="D48" s="8" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="E48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>729</v>
+        <v>737</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>730</v>
+        <v>738</v>
       </c>
       <c r="D49" s="8" t="s">
-        <v>731</v>
+        <v>739</v>
       </c>
       <c r="E49" s="10"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>732</v>
+        <v>740</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>733</v>
+        <v>741</v>
       </c>
       <c r="D50" s="8" t="s">
-        <v>734</v>
+        <v>742</v>
       </c>
       <c r="E50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>735</v>
+        <v>743</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>736</v>
+        <v>744</v>
       </c>
       <c r="D51" s="8" t="s">
-        <v>737</v>
+        <v>745</v>
       </c>
       <c r="E51" s="10"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>738</v>
+        <v>746</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>739</v>
+        <v>747</v>
       </c>
       <c r="D52" s="8" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="E52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>741</v>
+        <v>749</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>742</v>
+        <v>750</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="E53" s="10"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>743</v>
+        <v>751</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>744</v>
+        <v>752</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="E54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>745</v>
+        <v>753</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>746</v>
+        <v>754</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>747</v>
+        <v>755</v>
       </c>
       <c r="E55" s="10"/>
     </row>
     <row r="56" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>748</v>
+        <v>756</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>749</v>
+        <v>757</v>
       </c>
       <c r="D56" s="8" t="s">
-        <v>750</v>
+        <v>758</v>
       </c>
       <c r="E56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>751</v>
+        <v>759</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>752</v>
+        <v>760</v>
       </c>
       <c r="D57" s="8" t="s">
-        <v>753</v>
+        <v>761</v>
       </c>
       <c r="E57" s="10"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>754</v>
+        <v>762</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>755</v>
+        <v>763</v>
       </c>
       <c r="D58" s="8" t="s">
-        <v>756</v>
+        <v>764</v>
       </c>
       <c r="E58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>757</v>
+        <v>765</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>758</v>
+        <v>766</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="E59" s="10"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>759</v>
+        <v>767</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>760</v>
+        <v>768</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>740</v>
+        <v>748</v>
       </c>
       <c r="E60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>761</v>
+        <v>769</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>762</v>
+        <v>770</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>763</v>
+        <v>771</v>
       </c>
       <c r="E61" s="10"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>764</v>
+        <v>772</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>765</v>
+        <v>773</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>766</v>
+        <v>774</v>
       </c>
       <c r="E62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>767</v>
+        <v>775</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>768</v>
+        <v>776</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>769</v>
+        <v>777</v>
       </c>
       <c r="E63" s="10"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>770</v>
+        <v>778</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>771</v>
+        <v>779</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>726</v>
+        <v>734</v>
       </c>
       <c r="E64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>772</v>
+        <v>780</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>773</v>
+        <v>781</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>774</v>
+        <v>782</v>
       </c>
       <c r="E65" s="10"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>775</v>
+        <v>783</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>776</v>
+        <v>784</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>747</v>
+        <v>755</v>
       </c>
       <c r="E66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>777</v>
+        <v>785</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>778</v>
+        <v>786</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="E67" s="10"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>779</v>
+        <v>787</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>780</v>
+        <v>788</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>781</v>
+        <v>789</v>
       </c>
       <c r="E68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>782</v>
+        <v>790</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>783</v>
+        <v>791</v>
       </c>
       <c r="D69" s="8" t="s">
-        <v>784</v>
+        <v>792</v>
       </c>
       <c r="E69" s="10"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B70" s="7" t="s">
-        <v>785</v>
+        <v>793</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>786</v>
+        <v>794</v>
       </c>
       <c r="D70" s="8" t="s">
-        <v>787</v>
+        <v>795</v>
       </c>
       <c r="E70" s="10"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B71" s="7" t="s">
-        <v>788</v>
+        <v>796</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>789</v>
+        <v>797</v>
       </c>
       <c r="D71" s="8" t="s">
-        <v>790</v>
+        <v>798</v>
       </c>
       <c r="E71" s="10"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B72" s="7" t="s">
-        <v>791</v>
+        <v>799</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>792</v>
+        <v>800</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>700</v>
+        <v>708</v>
       </c>
       <c r="E72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>793</v>
+        <v>801</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>794</v>
+        <v>802</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>795</v>
+        <v>803</v>
       </c>
       <c r="E73" s="10"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
-        <v>691</v>
+        <v>699</v>
       </c>
       <c r="B74" s="7" t="s">
-        <v>796</v>
+        <v>804</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>797</v>
+        <v>805</v>
       </c>
       <c r="D74" s="8" t="s">
-        <v>798</v>
+        <v>806</v>
       </c>
       <c r="E74" s="10"/>
     </row>
@@ -40895,19 +41695,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>799</v>
+        <v>807</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>602</v>
+        <v>610</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>800</v>
+        <v>808</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>801</v>
+        <v>809</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>802</v>
+        <v>810</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -40915,434 +41715,434 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>803</v>
+        <v>811</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>804</v>
+        <v>812</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>805</v>
+        <v>813</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>806</v>
+        <v>814</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>539</v>
+        <v>547</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>807</v>
+        <v>815</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>805</v>
+        <v>813</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>808</v>
+        <v>816</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>809</v>
+        <v>817</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>810</v>
+        <v>818</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>805</v>
+        <v>813</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>811</v>
+        <v>819</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>812</v>
+        <v>820</v>
       </c>
       <c r="B5" s="7" t="s">
+        <v>821</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>813</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>805</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>814</v>
+        <v>822</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>815</v>
+        <v>823</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>816</v>
+        <v>824</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>817</v>
+        <v>825</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>818</v>
+        <v>826</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>819</v>
+        <v>827</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>820</v>
+        <v>828</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>821</v>
+        <v>829</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>822</v>
+        <v>830</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>823</v>
+        <v>831</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>824</v>
+        <v>832</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>825</v>
+        <v>833</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>826</v>
+        <v>834</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>827</v>
+        <v>835</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>828</v>
+        <v>836</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>829</v>
+        <v>837</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>830</v>
+        <v>838</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>831</v>
+        <v>839</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>832</v>
+        <v>840</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>833</v>
+        <v>841</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>834</v>
+        <v>842</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>835</v>
+        <v>843</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>836</v>
+        <v>844</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>837</v>
+        <v>845</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>838</v>
+        <v>846</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>839</v>
+        <v>847</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>840</v>
+        <v>848</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>841</v>
+        <v>849</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>842</v>
+        <v>850</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>843</v>
+        <v>851</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>844</v>
+        <v>852</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>845</v>
+        <v>853</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>846</v>
+        <v>854</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>847</v>
+        <v>855</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>848</v>
+        <v>856</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>849</v>
+        <v>857</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>850</v>
+        <v>858</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>851</v>
+        <v>859</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>852</v>
+        <v>860</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>853</v>
+        <v>861</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>854</v>
+        <v>862</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>855</v>
+        <v>863</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>829</v>
+        <v>837</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>856</v>
+        <v>864</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>857</v>
+        <v>865</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>858</v>
+        <v>866</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>859</v>
+        <v>867</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>860</v>
+        <v>868</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>861</v>
+        <v>869</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>862</v>
+        <v>870</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>863</v>
+        <v>871</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>864</v>
+        <v>872</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>865</v>
+        <v>873</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>866</v>
+        <v>874</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>867</v>
+        <v>875</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>868</v>
+        <v>876</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>869</v>
+        <v>877</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>870</v>
+        <v>878</v>
       </c>
       <c r="F24" s="10"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>871</v>
+        <v>879</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>872</v>
+        <v>880</v>
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>873</v>
+        <v>881</v>
       </c>
       <c r="F25" s="10"/>
     </row>
     <row r="26" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>874</v>
+        <v>882</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>875</v>
+        <v>883</v>
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>876</v>
+        <v>884</v>
       </c>
       <c r="F26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>877</v>
+        <v>885</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>878</v>
+        <v>886</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>879</v>
+        <v>887</v>
       </c>
       <c r="F27" s="10"/>
     </row>
     <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>880</v>
+        <v>888</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>881</v>
+        <v>889</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="8" t="n">
@@ -41353,26 +42153,26 @@
     </row>
     <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>882</v>
+        <v>890</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>883</v>
+        <v>891</v>
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>858</v>
+        <v>866</v>
       </c>
       <c r="F29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>884</v>
+        <v>892</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>885</v>
+        <v>893</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="7" t="n">
@@ -41411,22 +42211,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>886</v>
+        <v>894</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>628</v>
+        <v>636</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>480</v>
+        <v>488</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>887</v>
+        <v>895</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>888</v>
+        <v>896</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>802</v>
+        <v>810</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -41434,115 +42234,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>889</v>
+        <v>897</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>890</v>
+        <v>898</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>891</v>
+        <v>899</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>892</v>
+        <v>900</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>893</v>
+        <v>901</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>894</v>
+        <v>902</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>895</v>
+        <v>903</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>896</v>
+        <v>904</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>897</v>
+        <v>905</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>898</v>
+        <v>906</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>899</v>
+        <v>907</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>900</v>
+        <v>908</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>901</v>
+        <v>909</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>902</v>
+        <v>910</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>903</v>
+        <v>911</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>904</v>
+        <v>912</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>905</v>
+        <v>913</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>906</v>
+        <v>914</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>907</v>
+        <v>915</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>908</v>
+        <v>916</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>909</v>
+        <v>917</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>910</v>
+        <v>918</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>911</v>
+        <v>919</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>912</v>
+        <v>920</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>913</v>
+        <v>921</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>914</v>
+        <v>922</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>915</v>
+        <v>923</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>916</v>
+        <v>924</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>917</v>
+        <v>925</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>918</v>
+        <v>926</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>919</v>
+        <v>927</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>920</v>
+        <v>928</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
beta v0.12.30: sticky note helper shields every 6s, at most 3 active (4 for elites)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -14878,6 +14878,40 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">秒替最近、沒有盾的敵人貼便利貼（同時最多 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">隻，精英 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">4 </t>
     </r>
     <r>
@@ -14886,7 +14920,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">秒替最近、沒有盾的敵人貼便利貼：</t>
+      <t xml:space="preserve">隻）：</t>
     </r>
     <r>
       <rPr>
@@ -14969,6 +15003,42 @@
       </rPr>
       <t xml:space="preserve">2.6
 stickEvery</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6
+maxNotes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3
+eliteMaxNotes</t>
     </r>
     <r>
       <rPr>
@@ -38860,7 +38930,7 @@
       </c>
       <c r="P10" s="10"/>
     </row>
-    <row r="11" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
         <v>434</v>
       </c>

</xml_diff>

<commit_message>
beta v0.12.31: guaranteed enemy variety, bigger act 3 arenas with new cover, ink rain covers wall edges
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -22425,26 +22425,26 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">16
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">落點範圍：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">[9, 5.2]
+edge</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">：</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">0.4
 </t>
     </r>
     <r>

</xml_diff>

<commit_message>
v0.12.33: inertia scrolling for codex and weapon list, barrel blast kill achievement
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1343" uniqueCount="929">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1347" uniqueCount="932">
   <si>
     <r>
       <rPr>
@@ -30285,6 +30285,86 @@
         <charset val="1"/>
       </rPr>
       <t xml:space="preserve">250</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">一桶天下</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">用油桶爆炸累計炸倒 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">個敵人</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">40</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">／</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">80</t>
     </r>
   </si>
   <si>
@@ -40623,7 +40703,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -41418,7 +41498,7 @@
         <v>750</v>
       </c>
       <c r="D53" s="8" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
       <c r="E53" s="10"/>
     </row>
@@ -41427,32 +41507,32 @@
         <v>699</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="D54" s="8" t="s">
-        <v>708</v>
+        <v>748</v>
       </c>
       <c r="E54" s="10"/>
     </row>
-    <row r="55" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
         <v>699</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>755</v>
+        <v>708</v>
       </c>
       <c r="E55" s="10"/>
     </row>
-    <row r="56" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
         <v>699</v>
       </c>
@@ -41467,7 +41547,7 @@
       </c>
       <c r="E56" s="10"/>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="27.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
         <v>699</v>
       </c>
@@ -41508,7 +41588,7 @@
         <v>766</v>
       </c>
       <c r="D59" s="8" t="s">
-        <v>708</v>
+        <v>767</v>
       </c>
       <c r="E59" s="10"/>
     </row>
@@ -41517,13 +41597,13 @@
         <v>699</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>748</v>
+        <v>708</v>
       </c>
       <c r="E60" s="10"/>
     </row>
@@ -41532,13 +41612,13 @@
         <v>699</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>771</v>
+        <v>748</v>
       </c>
       <c r="E61" s="10"/>
     </row>
@@ -41583,7 +41663,7 @@
         <v>779</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>734</v>
+        <v>780</v>
       </c>
       <c r="E64" s="10"/>
     </row>
@@ -41592,13 +41672,13 @@
         <v>699</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="D65" s="8" t="s">
-        <v>782</v>
+        <v>734</v>
       </c>
       <c r="E65" s="10"/>
     </row>
@@ -41613,7 +41693,7 @@
         <v>784</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>755</v>
+        <v>785</v>
       </c>
       <c r="E66" s="10"/>
     </row>
@@ -41622,13 +41702,13 @@
         <v>699</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="D67" s="8" t="s">
-        <v>708</v>
+        <v>758</v>
       </c>
       <c r="E67" s="10"/>
     </row>
@@ -41637,13 +41717,13 @@
         <v>699</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="D68" s="8" t="s">
-        <v>789</v>
+        <v>708</v>
       </c>
       <c r="E68" s="10"/>
     </row>
@@ -41703,7 +41783,7 @@
         <v>800</v>
       </c>
       <c r="D72" s="8" t="s">
-        <v>708</v>
+        <v>801</v>
       </c>
       <c r="E72" s="10"/>
     </row>
@@ -41712,13 +41792,13 @@
         <v>699</v>
       </c>
       <c r="B73" s="7" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="D73" s="8" t="s">
-        <v>803</v>
+        <v>708</v>
       </c>
       <c r="E73" s="10"/>
     </row>
@@ -41736,6 +41816,21 @@
         <v>806</v>
       </c>
       <c r="E74" s="10"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="7" t="s">
+        <v>699</v>
+      </c>
+      <c r="B75" s="7" t="s">
+        <v>807</v>
+      </c>
+      <c r="C75" s="7" t="s">
+        <v>808</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>809</v>
+      </c>
+      <c r="E75" s="10"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -41765,19 +41860,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>610</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>808</v>
+        <v>811</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>810</v>
+        <v>813</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>32</v>
@@ -41785,19 +41880,19 @@
     </row>
     <row r="2" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>811</v>
+        <v>814</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>812</v>
+        <v>815</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>813</v>
+        <v>816</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>814</v>
+        <v>817</v>
       </c>
       <c r="F2" s="10"/>
     </row>
@@ -41806,413 +41901,413 @@
         <v>547</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>815</v>
+        <v>818</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>813</v>
+        <v>816</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>816</v>
+        <v>819</v>
       </c>
       <c r="F3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>817</v>
+        <v>820</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>818</v>
+        <v>821</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>813</v>
+        <v>816</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="F4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>820</v>
+        <v>823</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>821</v>
+        <v>824</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>813</v>
+        <v>816</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>822</v>
+        <v>825</v>
       </c>
       <c r="F5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>823</v>
+        <v>826</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>824</v>
+        <v>827</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>825</v>
+        <v>828</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>826</v>
+        <v>829</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>827</v>
+        <v>830</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>828</v>
+        <v>831</v>
       </c>
       <c r="F7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>829</v>
+        <v>832</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>830</v>
+        <v>833</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
       <c r="F8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>832</v>
+        <v>835</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>833</v>
+        <v>836</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>834</v>
+        <v>837</v>
       </c>
       <c r="F9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>835</v>
+        <v>838</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>836</v>
+        <v>839</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>837</v>
+        <v>840</v>
       </c>
       <c r="F10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>838</v>
+        <v>841</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>839</v>
+        <v>842</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>840</v>
+        <v>843</v>
       </c>
       <c r="F11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>841</v>
+        <v>844</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>842</v>
+        <v>845</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>843</v>
+        <v>846</v>
       </c>
       <c r="F12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>844</v>
+        <v>847</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>845</v>
+        <v>848</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>846</v>
+        <v>849</v>
       </c>
       <c r="F13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>847</v>
+        <v>850</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>848</v>
+        <v>851</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>849</v>
+        <v>852</v>
       </c>
       <c r="F14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>850</v>
+        <v>853</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>851</v>
+        <v>854</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>852</v>
+        <v>855</v>
       </c>
       <c r="F15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>853</v>
+        <v>856</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>854</v>
+        <v>857</v>
       </c>
       <c r="C16" s="7"/>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>855</v>
+        <v>858</v>
       </c>
       <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>856</v>
+        <v>859</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>857</v>
+        <v>860</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>858</v>
+        <v>861</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>859</v>
+        <v>862</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>860</v>
+        <v>863</v>
       </c>
       <c r="C18" s="7"/>
       <c r="D18" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>861</v>
+        <v>864</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>862</v>
+        <v>865</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>863</v>
+        <v>866</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>837</v>
+        <v>840</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>864</v>
+        <v>867</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>865</v>
+        <v>868</v>
       </c>
       <c r="C20" s="7"/>
       <c r="D20" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>866</v>
+        <v>869</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>867</v>
+        <v>870</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>868</v>
+        <v>871</v>
       </c>
       <c r="C21" s="7"/>
       <c r="D21" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>869</v>
+        <v>872</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>870</v>
+        <v>873</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>871</v>
+        <v>874</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>872</v>
+        <v>875</v>
       </c>
       <c r="F22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>874</v>
+        <v>877</v>
       </c>
       <c r="C23" s="7"/>
       <c r="D23" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>875</v>
+        <v>878</v>
       </c>
       <c r="F23" s="10"/>
     </row>
     <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>876</v>
+        <v>879</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>877</v>
+        <v>880</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>878</v>
+        <v>881</v>
       </c>
       <c r="F24" s="10"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>879</v>
+        <v>882</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>880</v>
+        <v>883</v>
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>881</v>
+        <v>884</v>
       </c>
       <c r="F25" s="10"/>
     </row>
     <row r="26" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>883</v>
+        <v>886</v>
       </c>
       <c r="C26" s="7"/>
       <c r="D26" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>884</v>
+        <v>887</v>
       </c>
       <c r="F26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>885</v>
+        <v>888</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>886</v>
+        <v>889</v>
       </c>
       <c r="C27" s="7"/>
       <c r="D27" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>887</v>
+        <v>890</v>
       </c>
       <c r="F27" s="10"/>
     </row>
     <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>888</v>
+        <v>891</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>889</v>
+        <v>892</v>
       </c>
       <c r="C28" s="7"/>
       <c r="D28" s="8" t="n">
@@ -42223,26 +42318,26 @@
     </row>
     <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>890</v>
+        <v>893</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>891</v>
+        <v>894</v>
       </c>
       <c r="C29" s="7"/>
       <c r="D29" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>866</v>
+        <v>869</v>
       </c>
       <c r="F29" s="10"/>
     </row>
     <row r="30" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>892</v>
+        <v>895</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>893</v>
+        <v>896</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="7" t="n">
@@ -42281,7 +42376,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>894</v>
+        <v>897</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>636</v>
@@ -42290,13 +42385,13 @@
         <v>488</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>895</v>
+        <v>898</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>896</v>
+        <v>899</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>810</v>
+        <v>813</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>32</v>
@@ -42304,115 +42399,115 @@
     </row>
     <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>897</v>
+        <v>900</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>898</v>
+        <v>901</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>899</v>
+        <v>902</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>900</v>
+        <v>903</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>901</v>
+        <v>904</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>902</v>
+        <v>905</v>
       </c>
       <c r="G2" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>903</v>
+        <v>906</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>904</v>
+        <v>907</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>905</v>
+        <v>908</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>906</v>
+        <v>909</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>907</v>
+        <v>910</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>908</v>
+        <v>911</v>
       </c>
       <c r="G3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>909</v>
+        <v>912</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>910</v>
+        <v>913</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>911</v>
+        <v>914</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>912</v>
+        <v>915</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>913</v>
+        <v>916</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="G4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="162.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>916</v>
+        <v>919</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>917</v>
+        <v>920</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>920</v>
+        <v>923</v>
       </c>
       <c r="G5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>921</v>
+        <v>924</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>922</v>
+        <v>925</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>923</v>
+        <v>926</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>924</v>
+        <v>927</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>925</v>
+        <v>928</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
       <c r="G6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>928</v>
+        <v>931</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>

</xml_diff>

<commit_message>
v0.12.34: slower pen fire rate, crayon damage 6/10/30
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -18610,7 +18610,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">28</t>
+      <t xml:space="preserve">30</t>
     </r>
     <r>
       <rPr>
@@ -18678,7 +18678,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">5</t>
+      <t xml:space="preserve">6</t>
     </r>
   </si>
   <si>
@@ -39596,7 +39596,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="8" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="H2" s="8" t="n">
         <v>12</v>
@@ -39615,7 +39615,7 @@
       </c>
       <c r="M2" s="7" t="n">
         <f aca="false">ROUND(E2*F2/G2,1)</f>
-        <v>83.3</v>
+        <v>66.7</v>
       </c>
       <c r="N2" s="7"/>
       <c r="O2" s="10"/>
@@ -39862,7 +39862,7 @@
         <v>512</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F8" s="8" t="n">
         <v>1</v>
@@ -39887,7 +39887,7 @@
       </c>
       <c r="M8" s="7" t="n">
         <f aca="false">ROUND(E8*F8/G8,1)</f>
-        <v>33.3</v>
+        <v>40</v>
       </c>
       <c r="N8" s="7" t="s">
         <v>513</v>

</xml_diff>

<commit_message>
v0.12.35: rename slingshot to Ink Bow, full-charge hit restores 2 ink
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -12436,7 +12436,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">。使用圓規或橡皮筋彈弓時不會出現（抽到直接棄掉）。</t>
+      <t xml:space="preserve">。使用圓規或墨弓時不會出現（抽到直接棄掉）。</t>
     </r>
   </si>
   <si>
@@ -18685,7 +18685,7 @@
     <t xml:space="preserve">slingshot</t>
   </si>
   <si>
-    <t xml:space="preserve">橡皮筋彈弓</t>
+    <t xml:space="preserve">墨弓</t>
   </si>
   <si>
     <t xml:space="preserve">蓄力穿透・無彈匣</t>

</xml_diff>

<commit_message>
v0.12.36: mechanical pencil damage 6
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -39634,7 +39634,7 @@
         <v>494</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>1</v>
@@ -39659,7 +39659,7 @@
       </c>
       <c r="M3" s="7" t="n">
         <f aca="false">ROUND(E3*F3/G3,1)</f>
-        <v>55.6</v>
+        <v>66.7</v>
       </c>
       <c r="N3" s="7"/>
       <c r="O3" s="10"/>

</xml_diff>

<commit_message>
v0.12.37: sticky helper sticks on arrival then every 4s, compass cooldown 1.2s
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181rgZBKpvoJcfkcsVzxNzL
</commit_message>
<xml_diff>
--- a/數值表.xlsx
+++ b/數值表.xlsx
@@ -14869,16 +14869,16 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【貼紙盾】每 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">6 </t>
+      <t xml:space="preserve">【貼紙盾】一出現就先貼一張，之後每 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4 </t>
     </r>
     <r>
       <rPr>
@@ -15019,7 +15019,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">6
+      <t xml:space="preserve">4
 maxNotes</t>
     </r>
     <r>
@@ -18557,7 +18557,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.5 </t>
+      <t xml:space="preserve">1.2 </t>
     </r>
     <r>
       <rPr>
@@ -39822,7 +39822,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>454</v>
@@ -39841,7 +39841,7 @@
       </c>
       <c r="M7" s="7" t="n">
         <f aca="false">ROUND(E7*F7/G7,1)</f>
-        <v>13.3</v>
+        <v>16.7</v>
       </c>
       <c r="N7" s="7" t="s">
         <v>509</v>

</xml_diff>